<commit_message>
Match clubs with a state suffix only within their state in the gap list
Vasco-AC, Santa Cruz-AC, Portuguesa-RJ and Sampaio Corrêa-RJ had been
matched to the namesakes from other states; the gap list now has 162 clubs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ka8oG79CEjWqcKUePCHJKb
</commit_message>
<xml_diff>
--- a/data/brasil/clubes/clubes_faltando.xlsx
+++ b/data/brasil/clubes/clubes_faltando.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF154"/>
+  <dimension ref="A1:AF163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -697,24 +697,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>São Francisco-AC</t>
+          <t>Santa Cruz-AC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Palmeira dos Índios</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Rio Branco</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -724,24 +719,24 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>CSE</t>
+          <t>São Francisco-AC</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AL</t>
+          <t>AC</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Coruripe</t>
+          <t>Rio Branco</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -756,7 +751,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Coruripe</t>
+          <t>Vasco-AC</t>
         </is>
       </c>
     </row>
@@ -768,7 +763,12 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arapiraca</t>
+          <t>Palmeira dos Índios</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -778,12 +778,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Cruzeiro de Arapiraca</t>
+          <t>CSE</t>
         </is>
       </c>
     </row>
@@ -795,7 +795,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Murici</t>
+          <t>Coruripe</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -810,19 +810,19 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Murici SC</t>
+          <t>Coruripe</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Itacoatiara</t>
+          <t>Arapiraca</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -837,24 +837,19 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Itacoatiara</t>
+          <t>Cruzeiro de Arapiraca</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>AL</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Manaus</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Murici</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -864,12 +859,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Nacional</t>
+          <t>Murici SC</t>
         </is>
       </c>
     </row>
@@ -881,7 +876,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Parintins</t>
+          <t>Itacoatiara</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -896,7 +891,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Parintins</t>
+          <t>Itacoatiara</t>
         </is>
       </c>
     </row>
@@ -908,7 +903,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Manacapuru</t>
+          <t>Manaus</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -918,12 +918,12 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Princesa do Solimões</t>
+          <t>Nacional</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Manaus</t>
+          <t>Parintins</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -950,19 +950,19 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>São Raimundo-AM</t>
+          <t>Parintins</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Macapá</t>
+          <t>Manacapuru</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -977,19 +977,19 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Cristal</t>
+          <t>Princesa do Solimões</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AP</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Santana</t>
+          <t>Manaus</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Independente</t>
+          <t>São Raimundo-AM</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Macapá</t>
+          <t>Cristal</t>
         </is>
       </c>
     </row>
@@ -1043,12 +1043,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Macapá</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Santana</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1058,12 +1053,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Oratório</t>
+          <t>Independente</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1085,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>São José-AP</t>
+          <t>Macapá</t>
         </is>
       </c>
     </row>
@@ -1105,6 +1100,11 @@
           <t>Macapá</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>sim</t>
@@ -1112,29 +1112,24 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Ypiranga-AP</t>
+          <t>Oratório</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Alagoinhas</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Macapá</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1144,24 +1139,24 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Atlético de Alagoinhas</t>
+          <t>Santos-AP</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Feira de Santana</t>
+          <t>Macapá</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1176,19 +1171,19 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Bahia de Feira</t>
+          <t>São José-AP</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>AP</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Salvador</t>
+          <t>Macapá</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1203,7 +1198,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Galícia</t>
+          <t>Ypiranga-AP</t>
         </is>
       </c>
     </row>
@@ -1215,7 +1210,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Riachão do Jacuípe</t>
+          <t>Alagoinhas</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1235,7 +1230,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Jacuipense</t>
+          <t>Atlético de Alagoinhas</t>
         </is>
       </c>
     </row>
@@ -1247,12 +1242,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Porto Seguro</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Feira de Santana</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1262,51 +1252,56 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Porto</t>
+          <t>Bahia de Feira</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CE</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Salvador</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Atlético Cearense</t>
+          <t>Galícia</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Maranguape</t>
+          <t>Riachão do Jacuípe</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1316,24 +1311,29 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Maranguape</t>
+          <t>Jacuipense</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CE</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Quixadá</t>
+          <t>Porto Seguro</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1343,12 +1343,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Quixadá</t>
+          <t>Porto</t>
         </is>
       </c>
     </row>
@@ -1358,11 +1358,6 @@
           <t>CE</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Fortaleza</t>
-        </is>
-      </c>
       <c r="C29" t="inlineStr">
         <is>
           <t>D</t>
@@ -1370,7 +1365,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1380,19 +1375,19 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Tirol</t>
+          <t>Atlético Cearense</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Cruzeiro</t>
+          <t>Maranguape</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1407,24 +1402,19 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>ARUC</t>
+          <t>Maranguape</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Taguatinga</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Quixadá</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1434,24 +1424,29 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Brasiliense</t>
+          <t>Quixadá</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DF</t>
+          <t>CE</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Fortaleza</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1461,12 +1456,12 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Brasília</t>
+          <t>Tirol</t>
         </is>
       </c>
     </row>
@@ -1478,12 +1473,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Gama</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Cruzeiro</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1493,12 +1483,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Gama</t>
+          <t>ARUC</t>
         </is>
       </c>
     </row>
@@ -1510,7 +1500,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Paranoá</t>
+          <t>Taguatinga</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1520,12 +1515,12 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Paranoá</t>
+          <t>Brasiliense</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1547,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Real Brasília</t>
+          <t>Brasília</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1559,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Samambaia</t>
+          <t>Gama</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1574,12 +1574,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Samambaia</t>
+          <t>Gama</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Sobradinho</t>
+          <t>Paranoá</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1606,19 +1606,19 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Sobradinho</t>
+          <t>Paranoá</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Vila Velha</t>
+          <t>Brasília</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1633,19 +1633,19 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Capixaba</t>
+          <t>Real Brasília</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cariacica</t>
+          <t>Samambaia</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1660,19 +1660,19 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Desportiva Ferroviária</t>
+          <t>Samambaia</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>DF</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Castelo</t>
+          <t>Sobradinho</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1687,7 +1687,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Forte</t>
+          <t>Sobradinho</t>
         </is>
       </c>
     </row>
@@ -1699,12 +1699,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Águia Branca</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Vila Velha</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1714,12 +1709,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Real Noroeste</t>
+          <t>Capixaba</t>
         </is>
       </c>
     </row>
@@ -1731,7 +1726,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Venda Nova do Imigrante</t>
+          <t>Cariacica</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1746,7 +1741,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Rio Branco de Venda Nova</t>
+          <t>Desportiva Ferroviária</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1753,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Serra</t>
+          <t>Castelo</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1773,7 +1768,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Serra</t>
+          <t>Forte</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1780,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Vila Velha</t>
+          <t>Águia Branca</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1795,29 +1795,24 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Vilavelhense</t>
+          <t>Real Noroeste</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Ouvidor</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Venda Nova do Imigrante</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1827,24 +1822,24 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>ABECAT</t>
+          <t>Rio Branco de Venda Nova</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Anápolis</t>
+          <t>Serra</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1859,24 +1854,19 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Anapolina</t>
+          <t>Serra</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Catalão</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Vila Velha</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1886,24 +1876,29 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>CRAC</t>
+          <t>Vilavelhense</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Senador Canedo</t>
+          <t>Vitória</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1913,12 +1908,12 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Centro Oeste</t>
+          <t>Vitória-ES</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1925,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Inhumas</t>
+          <t>Ouvidor</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1950,7 +1945,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Inhumas</t>
+          <t>ABECAT</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1957,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Jataí</t>
+          <t>Anápolis</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1977,19 +1972,19 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Jataiense</t>
+          <t>Anapolina</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>São Luís</t>
+          <t>Catalão</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2009,19 +2004,19 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>IAPE</t>
+          <t>CRAC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Imperatriz</t>
+          <t>Senador Canedo</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2036,19 +2031,24 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>ITZ Sport</t>
+          <t>Centro Oeste</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Paço do Lumiar</t>
+          <t>Inhumas</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -2058,29 +2058,24 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Luminense</t>
+          <t>Inhumas</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>São Luís</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Jataí</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -2090,12 +2085,12 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Moto Club</t>
+          <t>Jataiense</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2102,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Tuntum</t>
+          <t>São Luís</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2117,29 +2117,24 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Tuntum</t>
+          <t>IAPE</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Betim</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Imperatriz</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2149,29 +2144,24 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Betim</t>
+          <t>ITZ Sport</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Governador Valadares</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Paço do Lumiar</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2181,24 +2171,29 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Democrata GV</t>
+          <t>Luminense</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Montes Claros</t>
+          <t>São Luís</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2208,24 +2203,24 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>North</t>
+          <t>Moto Club</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Patos de Minas</t>
+          <t>Tuntum</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2240,19 +2235,24 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>URT</t>
+          <t>Tuntum</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Bataguassu</t>
+          <t>Betim</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2262,24 +2262,29 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Bataguassu</t>
+          <t>Betim</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Aquidauana</t>
+          <t>Governador Valadares</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2289,24 +2294,24 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>CRA</t>
+          <t>Democrata GV</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Corumbá</t>
+          <t>Montes Claros</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2321,19 +2326,19 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Corumbaense</t>
+          <t>North</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>Patos de Minas</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -2348,7 +2353,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>URT</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2365,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Dourados</t>
+          <t>Bataguassu</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2375,7 +2380,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Dourados</t>
+          <t>Bataguassu</t>
         </is>
       </c>
     </row>
@@ -2385,24 +2390,24 @@
           <t>MS</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>D</t>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Aquidauana</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>FC Pantanal</t>
+          <t>CRA</t>
         </is>
       </c>
     </row>
@@ -2414,7 +2419,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Ivinhema</t>
+          <t>Corumbá</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2429,7 +2434,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>Ivinhema</t>
+          <t>Corumbaense</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2446,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Naviraí</t>
+          <t>Costa Rica</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2456,7 +2461,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>Naviraiense</t>
+          <t>Costa Rica</t>
         </is>
       </c>
     </row>
@@ -2468,7 +2473,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Campo Grande</t>
+          <t>Dourados</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2476,11 +2481,6 @@
           <t>sim</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>verificar: é o mesmo que FC Pantanal?</t>
-        </is>
-      </c>
       <c r="F68" t="inlineStr">
         <is>
           <t>estadual</t>
@@ -2488,7 +2488,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>Pantanal</t>
+          <t>Dourados</t>
         </is>
       </c>
     </row>
@@ -2498,36 +2498,36 @@
           <t>MS</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Rio Brilhante</t>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>Águia Negra</t>
+          <t>FC Pantanal</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Chapada dos Guimarães</t>
+          <t>Ivinhema</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2542,19 +2542,19 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Chapada</t>
+          <t>Ivinhema</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Nova Mutum</t>
+          <t>Naviraí</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2569,24 +2569,19 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Nova Mutum</t>
+          <t>Naviraiense</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Várzea Grande</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Campo Grande</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2594,31 +2589,31 @@
           <t>sim</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>verificar: é o mesmo que FC Pantanal?</t>
+        </is>
+      </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Operário VG</t>
+          <t>Pantanal</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MT</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Primavera do Leste</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Rio Brilhante</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2628,12 +2623,12 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Primavera</t>
+          <t>Águia Negra</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2640,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Sinop</t>
+          <t>Chapada dos Guimarães</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2660,7 +2655,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Sport Sinop</t>
+          <t>Chapada</t>
         </is>
       </c>
     </row>
@@ -2672,12 +2667,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Rondonópolis</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Nova Mutum</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2687,12 +2677,12 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>União Rondonópolis</t>
+          <t>Nova Mutum</t>
         </is>
       </c>
     </row>
@@ -2707,6 +2697,11 @@
           <t>Várzea Grande</t>
         </is>
       </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
       <c r="D76" t="inlineStr">
         <is>
           <t>sim</t>
@@ -2714,24 +2709,29 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Várzea Grande</t>
+          <t>Operário VG</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Belterra</t>
+          <t>Primavera do Leste</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -2741,24 +2741,24 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>Amazônia</t>
+          <t>Primavera</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Cametá</t>
+          <t>Sinop</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2773,19 +2773,24 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Cametá</t>
+          <t>Sport Sinop</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Capitão Poço</t>
+          <t>Rondonópolis</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2795,24 +2800,24 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>Capitão Poço</t>
+          <t>União Rondonópolis</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>PA</t>
+          <t>MT</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Castanhal</t>
+          <t>Várzea Grande</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2827,7 +2832,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Castanhal</t>
+          <t>Várzea Grande</t>
         </is>
       </c>
     </row>
@@ -2839,7 +2844,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Belém</t>
+          <t>Belterra</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2854,7 +2859,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>Santa Rosa</t>
+          <t>Amazônia</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2871,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Bragança</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2881,7 +2886,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>São Francisco-PA</t>
+          <t>Bragantino-PA</t>
         </is>
       </c>
     </row>
@@ -2893,7 +2898,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Santarém</t>
+          <t>Cametá</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -2908,19 +2913,19 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>São Raimundo-PA</t>
+          <t>Cametá</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Cajazeiras</t>
+          <t>Capitão Poço</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2935,19 +2940,19 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>Atlético de Cajazeiras</t>
+          <t>Capitão Poço</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Campina Grande</t>
+          <t>Castanhal</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2962,19 +2967,19 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>Campinense</t>
+          <t>Castanhal</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Sapé</t>
+          <t>Belém</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2989,19 +2994,19 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>Confiança de Sapé</t>
+          <t>Santa Rosa</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Patos</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3016,19 +3021,19 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>Esporte de Patos</t>
+          <t>São Francisco-PA</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>PB</t>
+          <t>PA</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Patos</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3043,7 +3048,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>Nacional de Patos</t>
+          <t>São Raimundo-PA</t>
         </is>
       </c>
     </row>
@@ -3055,7 +3060,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Pombal</t>
+          <t>Cajazeiras</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3070,7 +3075,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>Pombal</t>
+          <t>Atlético de Cajazeiras</t>
         </is>
       </c>
     </row>
@@ -3085,11 +3090,6 @@
           <t>Campina Grande</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
       <c r="D90" t="inlineStr">
         <is>
           <t>sim</t>
@@ -3097,24 +3097,24 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>Serra Branca</t>
+          <t>Campinense</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Goiana</t>
+          <t>Sapé</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3122,11 +3122,6 @@
           <t>sim</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr">
-        <is>
-          <t>verificar: é o mesmo que Decisão Goiana?</t>
-        </is>
-      </c>
       <c r="F91" t="inlineStr">
         <is>
           <t>estadual</t>
@@ -3134,46 +3129,46 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>Decisão</t>
+          <t>Confiança de Sapé</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>PE</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>PB</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Patos</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>Decisão Goiana</t>
+          <t>Esporte de Patos</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Jaboatão dos Guararapes</t>
+          <t>Patos</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3188,24 +3183,19 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Jaguar</t>
+          <t>Nacional de Patos</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Bonito</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Pombal</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3215,24 +3205,29 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>Maguary</t>
+          <t>Pombal</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>PB</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Vitória de Santo Antão</t>
+          <t>Campina Grande</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3242,24 +3237,24 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>Vitória das Tabocas</t>
+          <t>Serra Branca</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Teresina</t>
+          <t>Goiana</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3267,6 +3262,11 @@
           <t>sim</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>verificar: é o mesmo que Decisão Goiana?</t>
+        </is>
+      </c>
       <c r="F96" t="inlineStr">
         <is>
           <t>estadual</t>
@@ -3274,46 +3274,46 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>Atlético Piauiense</t>
+          <t>Decisão</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PI</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Floriano</t>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>Corisabbá</t>
+          <t>Decisão Goiana</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Oeiras</t>
+          <t>Jaboatão dos Guararapes</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3328,19 +3328,19 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>Oeirense</t>
+          <t>Jaguar</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Teresina</t>
+          <t>Bonito</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -3360,19 +3360,19 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>Piauí</t>
+          <t>Maguary</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Teresina</t>
+          <t>Vitória de Santo Antão</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -3387,19 +3387,19 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Teresina</t>
+          <t>Vitória das Tabocas</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Campo Largo</t>
+          <t>Teresina</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3414,19 +3414,19 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Andraus</t>
+          <t>Atlético Piauiense</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Cascavel</t>
+          <t>Floriano</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -3434,11 +3434,6 @@
           <t>sim</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>verificar: é o mesmo que FC Cascavel (já na planilha)?</t>
-        </is>
-      </c>
       <c r="F102" t="inlineStr">
         <is>
           <t>estadual</t>
@@ -3446,19 +3441,24 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>Cascavel</t>
+          <t>Corisabbá</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Foz do Iguaçu</t>
+          <t>Teresina</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3468,24 +3468,24 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>Foz do Iguaçu</t>
+          <t>Fluminense-PI</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Maringá</t>
+          <t>Oeiras</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -3500,14 +3500,19 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Galo Maringá</t>
+          <t>Oeirense</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PI</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Teresina</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -3517,7 +3522,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -3527,19 +3532,19 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>PSTC/São Joseense</t>
+          <t>Piauí</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>PI</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>São José dos Pinhais</t>
+          <t>Teresina</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -3547,11 +3552,6 @@
           <t>sim</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>verificar: é o mesmo que PSTC/São Joseense?</t>
-        </is>
-      </c>
       <c r="F106" t="inlineStr">
         <is>
           <t>estadual</t>
@@ -3559,46 +3559,46 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>São Joseense</t>
+          <t>Teresina</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>RJ</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Campo Largo</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>América-RJ</t>
+          <t>Andraus</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
+          <t>Cascavel</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -3606,6 +3606,11 @@
           <t>sim</t>
         </is>
       </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>verificar: é o mesmo que FC Cascavel (já na planilha)?</t>
+        </is>
+      </c>
       <c r="F108" t="inlineStr">
         <is>
           <t>estadual</t>
@@ -3613,24 +3618,19 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>Bangu</t>
+          <t>Cascavel</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>RJ</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Rio de Janeiro</t>
-        </is>
-      </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Foz do Iguaçu</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -3640,24 +3640,24 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>Madureira</t>
+          <t>Foz do Iguaçu</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Ceará-Mirim</t>
+          <t>Maringá</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -3672,19 +3672,14 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Globo</t>
+          <t>Galo Maringá</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>RN</t>
-        </is>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Tibau do Sul</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -3694,7 +3689,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -3704,73 +3699,78 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Laguna</t>
+          <t>PSTC/São Joseense</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>RN</t>
-        </is>
-      </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>São José dos Pinhais</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>verificar: é o mesmo que PSTC/São Joseense?</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Parnamirim/ABC-D</t>
+          <t>São Joseense</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>RN</t>
-        </is>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Mossoró</t>
+          <t>RJ</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>Potiguar de Mossoró</t>
+          <t>América-RJ</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Currais Novos</t>
+          <t>Rio de Janeiro</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -3785,19 +3785,24 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>Potyguar Seridoense</t>
+          <t>Bangu</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>RN</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Parnamirim</t>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -3807,24 +3812,29 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>QFC</t>
+          <t>Madureira</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Porto Velho</t>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -3834,24 +3844,29 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Barcelona-RO</t>
+          <t>Portuguesa-RJ</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RJ</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Porto Velho</t>
+          <t>Saquarema</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3861,29 +3876,24 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>Genus</t>
+          <t>Sampaio Corrêa-RJ</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Rolim de Moura</t>
-        </is>
-      </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Ceará-Mirim</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3893,24 +3903,29 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>Guaporé</t>
+          <t>Globo</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Ji-Paraná</t>
+          <t>Tibau do Sul</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -3920,51 +3935,51 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>Ji-Paraná</t>
+          <t>Laguna</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>RO</t>
-        </is>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>Porto Velho</t>
+          <t>RN</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>Rondoniense</t>
+          <t>Parnamirim/ABC-D</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>RO</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Cacoal</t>
+          <t>Mossoró</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -3979,19 +3994,19 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>União Cacoalense</t>
+          <t>Potiguar de Mossoró</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Boa Vista</t>
+          <t>Currais Novos</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -4006,19 +4021,19 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>Atlético Roraima</t>
+          <t>Potyguar Seridoense</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RN</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Boa Vista</t>
+          <t>Parnamirim</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -4033,24 +4048,19 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>Baré</t>
+          <t>QFC</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Boa Vista</t>
-        </is>
-      </c>
-      <c r="C124" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Porto Velho</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -4060,24 +4070,24 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Monte Roraima</t>
+          <t>Barcelona-RO</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Mucajaí</t>
+          <t>Porto Velho</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -4092,19 +4102,24 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>Progresso</t>
+          <t>Genus</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Boa Vista</t>
+          <t>Rolim de Moura</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -4114,24 +4129,24 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>Rio Negro-RR</t>
+          <t>Guaporé</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Boa Vista</t>
+          <t>Ji-Paraná</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -4146,24 +4161,19 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>River-RR</t>
+          <t>Ji-Paraná</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>RR</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Boa Vista</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Porto Velho</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -4173,24 +4183,24 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>São Raimundo-RR</t>
+          <t>Rondoniense</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RO</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Santa Cruz do Sul</t>
+          <t>Cacoal</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -4205,19 +4215,19 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Avenida</t>
+          <t>União Cacoalense</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Santa Maria</t>
+          <t>Boa Vista</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -4232,19 +4242,19 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>Internacional de Santa Maria</t>
+          <t>Atlético Roraima</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Porto Alegre</t>
+          <t>Boa Vista</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -4259,19 +4269,24 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>Monsoon</t>
+          <t>Baré</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Novo Hamburgo</t>
+          <t>Boa Vista</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -4281,51 +4296,51 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>Novo Hamburgo</t>
+          <t>Monte Roraima</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>RR</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Boa Vista</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>Blumenau</t>
+          <t>Náutico-RR</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Camboriú</t>
+          <t>Mucajaí</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -4340,19 +4355,19 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>Camboriú</t>
+          <t>Progresso</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Brusque</t>
+          <t>Boa Vista</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -4367,19 +4382,19 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>Carlos Renaux</t>
+          <t>Rio Negro-RR</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Concórdia</t>
+          <t>Boa Vista</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -4394,19 +4409,19 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>Concórdia</t>
+          <t>River-RR</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RR</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Rio do Sul</t>
+          <t>Boa Vista</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -4426,19 +4441,19 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Santa Catarina</t>
+          <t>São Raimundo-RR</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Propriá</t>
+          <t>Santa Cruz do Sul</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
@@ -4453,19 +4468,19 @@
       </c>
       <c r="G138" t="inlineStr">
         <is>
-          <t>América de Propriá</t>
+          <t>Avenida</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Nossa Senhora da Glória</t>
+          <t>Santa Maria</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -4480,19 +4495,19 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Atlético Gloriense</t>
+          <t>Internacional de Santa Maria</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Aracaju</t>
+          <t>Porto Alegre</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -4507,19 +4522,19 @@
       </c>
       <c r="G140" t="inlineStr">
         <is>
-          <t>Desportiva Aracaju</t>
+          <t>Monsoon</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Nossa Senhora das Dores</t>
+          <t>Novo Hamburgo</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -4534,46 +4549,46 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>Dorense</t>
+          <t>Novo Hamburgo</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>SE</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>Barra dos Coqueiros</t>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>não</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>Falcon</t>
+          <t>Blumenau</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Porto da Folha</t>
+          <t>Camboriú</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -4588,19 +4603,19 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>Guarany de Porto da Folha</t>
+          <t>Camboriú</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Capivari</t>
+          <t>Brusque</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
@@ -4615,24 +4630,19 @@
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>Capivariano</t>
+          <t>Carlos Renaux</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Bauru</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Concórdia</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -4642,24 +4652,29 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>Noroeste</t>
+          <t>Concórdia</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Indaiatuba</t>
+          <t>Rio do Sul</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>D</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
@@ -4669,29 +4684,24 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>estadual</t>
+          <t>D</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>Primavera-SP</t>
+          <t>Santa Catarina</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Rio Claro</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Propriá</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -4701,56 +4711,51 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>Velo Clube</t>
+          <t>América de Propriá</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>SE</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Nossa Senhora da Glória</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>não</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>XV de Piracicaba</t>
+          <t>Atlético Gloriense</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Araguaína</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>D</t>
+          <t>Aracaju</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
@@ -4760,24 +4765,24 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>estadual</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>Araguaína</t>
+          <t>Desportiva Aracaju</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Cachoeirinha</t>
+          <t>Nossa Senhora das Dores</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -4792,19 +4797,19 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>Bela Vista</t>
+          <t>Dorense</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Palmas</t>
+          <t>Barra dos Coqueiros</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
@@ -4819,19 +4824,19 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>Capital-TO</t>
+          <t>Falcon</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Guaraí</t>
+          <t>Porto da Folha</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
@@ -4846,19 +4851,19 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>Guaraí</t>
+          <t>Guarany de Porto da Folha</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>TO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Gurupi</t>
+          <t>Capivari</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
@@ -4873,32 +4878,290 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>Gurupi</t>
+          <t>Capivariano</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Bauru</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Noroeste</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Indaiatuba</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>estadual</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Primavera-SP</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Rio Claro</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Velo Clube</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>não</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>XV de Piracicaba</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
           <t>TO</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Araguaína</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Araguaína</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Cachoeirinha</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>estadual</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Bela Vista</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>
       </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>sim</t>
-        </is>
-      </c>
-      <c r="F154" t="inlineStr">
-        <is>
-          <t>estadual</t>
-        </is>
-      </c>
-      <c r="G154" t="inlineStr">
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>estadual</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Capital-TO</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Guaraí</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>estadual</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Guaraí</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Gurupi</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>estadual</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Gurupi</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>TO</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Palmas</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>sim</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>estadual</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
         <is>
           <t>Palmas</t>
         </is>

</xml_diff>

<commit_message>
Listas times real, uniforme, patrocionio  2026 atualizado
</commit_message>
<xml_diff>
--- a/data/brasil/clubes/clubes_faltando.xlsx
+++ b/data/brasil/clubes/clubes_faltando.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faltando" sheetId="1" r:id="Rd880d0ae0a594ba3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA" sheetId="2" r:id="R2c05f6151c004c4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faltando" sheetId="1" r:id="R2112614f5c7441e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LEIA" sheetId="2" r:id="Ra054c0b968754f44"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10144,21 +10144,23 @@
         <x:v>RN</x:v>
       </x:c>
       <x:c r="B116" t="str">
-        <x:v>Mossoró</x:v>
+        <x:v>Parnamirim</x:v>
       </x:c>
       <x:c r="C116"/>
       <x:c r="D116" t="str">
-        <x:v>sim</x:v>
-      </x:c>
-      <x:c r="E116"/>
+        <x:v>não (desistiu)</x:v>
+      </x:c>
+      <x:c r="E116" t="str">
+        <x:v>Clube distinto do ABC. Confirmou inscrição na 2ª divisão potiguar de 2026, mas desistiu em 27/08/2026 antes do início da competição. Fonte: https://fnf.org.br/campeonato-potiguar-segunda-divisao-2026-cinco-clubes-disputarao-a-taca-a-partir-de-7-de-outubro</x:v>
+      </x:c>
       <x:c r="F116" t="str">
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G116" t="str">
-        <x:v>Potiguar de Mossoró</x:v>
+        <x:v>Parnamirim</x:v>
       </x:c>
       <x:c r="H116" t="str">
-        <x:v>potiguar_de_mossoro.png</x:v>
+        <x:v>parnamirim.png</x:v>
       </x:c>
       <x:c r="I116" t="str">
         <x:v>PNG</x:v>
@@ -10171,54 +10173,52 @@
       <x:c r="M116" t="n">
         <x:v>2026</x:v>
       </x:c>
-      <x:c r="N116" t="str">
-        <x:v>Football Kit Archive</x:v>
-      </x:c>
+      <x:c r="N116"/>
       <x:c r="O116"/>
       <x:c r="P116" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Potiguar+de+Mossor%C3%B3%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=%22Parnamirim+Sport+Clube%22+uniforme+2026</x:v>
       </x:c>
       <x:c r="Q116" t="str">
-        <x:v>PENDENTE DE FOTO DIRETA</x:v>
+        <x:v>SEM REFERÊNCIA 2026 CONFIRMADA</x:v>
       </x:c>
       <x:c r="R116" t="str">
-        <x:v>Vermelho / Branco</x:v>
+        <x:v>Azul / Amarelo</x:v>
       </x:c>
       <x:c r="S116" t="str">
-        <x:v>#D2232A / #FFFFFF</x:v>
+        <x:v>#0057B8 / #FFD100</x:v>
       </x:c>
       <x:c r="T116" t="str">
-        <x:v>210,35,42 / 255,255,255</x:v>
+        <x:v>0,87,184 / 255,209,0</x:v>
       </x:c>
       <x:c r="U116" t="str">
-        <x:v>Vermelho</x:v>
+        <x:v>Azul</x:v>
       </x:c>
       <x:c r="V116" t="str">
-        <x:v>#D2232A</x:v>
+        <x:v>#0057B8</x:v>
       </x:c>
       <x:c r="W116" t="str">
-        <x:v>210,35,42</x:v>
+        <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="X116" t="str">
-        <x:v>Branco</x:v>
+        <x:v>Amarelo</x:v>
       </x:c>
       <x:c r="Y116" t="str">
-        <x:v>#FFFFFF</x:v>
+        <x:v>#FFD100</x:v>
       </x:c>
       <x:c r="Z116" t="str">
-        <x:v>255,255,255</x:v>
+        <x:v>255,209,0</x:v>
       </x:c>
       <x:c r="AA116"/>
       <x:c r="AB116"/>
       <x:c r="AC116"/>
       <x:c r="AD116" t="str">
-        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+        <x:v>cores históricas do clube; fonte: https://www.rsssf.org/colours/brazil.html</x:v>
       </x:c>
       <x:c r="AE116" t="str">
-        <x:v>Potiguar de Mossoró</x:v>
+        <x:v>Parnamirim</x:v>
       </x:c>
       <x:c r="AF116" t="str">
-        <x:v>Associação Cultural e Desportiva Potiguar</x:v>
+        <x:v>Parnamirim Sport Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="117">
@@ -10226,7 +10226,7 @@
         <x:v>RN</x:v>
       </x:c>
       <x:c r="B117" t="str">
-        <x:v>Currais Novos</x:v>
+        <x:v>Mossoró</x:v>
       </x:c>
       <x:c r="C117"/>
       <x:c r="D117" t="str">
@@ -10237,10 +10237,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G117" t="str">
-        <x:v>Potyguar Seridoense</x:v>
+        <x:v>Potiguar de Mossoró</x:v>
       </x:c>
       <x:c r="H117" t="str">
-        <x:v>potyguar_seridoense.png</x:v>
+        <x:v>potiguar_de_mossoro.png</x:v>
       </x:c>
       <x:c r="I117" t="str">
         <x:v>PNG</x:v>
@@ -10258,19 +10258,19 @@
       </x:c>
       <x:c r="O117"/>
       <x:c r="P117" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Potyguar+Seridoense%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Potiguar+de+Mossor%C3%B3%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q117" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R117" t="str">
-        <x:v>Vermelho / Azul / Branco</x:v>
+        <x:v>Vermelho / Branco</x:v>
       </x:c>
       <x:c r="S117" t="str">
-        <x:v>#D2232A / #0057B8 / #FFFFFF</x:v>
+        <x:v>#D2232A / #FFFFFF</x:v>
       </x:c>
       <x:c r="T117" t="str">
-        <x:v>210,35,42 / 0,87,184 / 255,255,255</x:v>
+        <x:v>210,35,42 / 255,255,255</x:v>
       </x:c>
       <x:c r="U117" t="str">
         <x:v>Vermelho</x:v>
@@ -10282,31 +10282,25 @@
         <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="X117" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Branco</x:v>
       </x:c>
       <x:c r="Y117" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#FFFFFF</x:v>
       </x:c>
       <x:c r="Z117" t="str">
-        <x:v>0,87,184</x:v>
-      </x:c>
-      <x:c r="AA117" t="str">
-        <x:v>Branco</x:v>
-      </x:c>
-      <x:c r="AB117" t="str">
-        <x:v>#FFFFFF</x:v>
-      </x:c>
-      <x:c r="AC117" t="str">
         <x:v>255,255,255</x:v>
       </x:c>
+      <x:c r="AA117"/>
+      <x:c r="AB117"/>
+      <x:c r="AC117"/>
       <x:c r="AD117" t="str">
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE117" t="str">
-        <x:v>Potyguar Seridoense</x:v>
+        <x:v>Potiguar de Mossoró</x:v>
       </x:c>
       <x:c r="AF117" t="str">
-        <x:v>Associação Cultural e Desportiva Potyguar Seridoense</x:v>
+        <x:v>Associação Cultural e Desportiva Potiguar</x:v>
       </x:c>
     </x:row>
     <x:row r="118">
@@ -10314,7 +10308,7 @@
         <x:v>RN</x:v>
       </x:c>
       <x:c r="B118" t="str">
-        <x:v>Parnamirim</x:v>
+        <x:v>Currais Novos</x:v>
       </x:c>
       <x:c r="C118"/>
       <x:c r="D118" t="str">
@@ -10325,10 +10319,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G118" t="str">
-        <x:v>QFC</x:v>
+        <x:v>Potyguar Seridoense</x:v>
       </x:c>
       <x:c r="H118" t="str">
-        <x:v>qfc.png</x:v>
+        <x:v>potyguar_seridoense.png</x:v>
       </x:c>
       <x:c r="I118" t="str">
         <x:v>PNG</x:v>
@@ -10346,57 +10340,63 @@
       </x:c>
       <x:c r="O118"/>
       <x:c r="P118" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22QFC%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Potyguar+Seridoense%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q118" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R118" t="str">
-        <x:v>Azul / Branco</x:v>
+        <x:v>Vermelho / Azul / Branco</x:v>
       </x:c>
       <x:c r="S118" t="str">
-        <x:v>#0057B8 / #FFFFFF</x:v>
+        <x:v>#D2232A / #0057B8 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T118" t="str">
-        <x:v>0,87,184 / 255,255,255</x:v>
+        <x:v>210,35,42 / 0,87,184 / 255,255,255</x:v>
       </x:c>
       <x:c r="U118" t="str">
+        <x:v>Vermelho</x:v>
+      </x:c>
+      <x:c r="V118" t="str">
+        <x:v>#D2232A</x:v>
+      </x:c>
+      <x:c r="W118" t="str">
+        <x:v>210,35,42</x:v>
+      </x:c>
+      <x:c r="X118" t="str">
         <x:v>Azul</x:v>
       </x:c>
-      <x:c r="V118" t="str">
+      <x:c r="Y118" t="str">
         <x:v>#0057B8</x:v>
       </x:c>
-      <x:c r="W118" t="str">
+      <x:c r="Z118" t="str">
         <x:v>0,87,184</x:v>
       </x:c>
-      <x:c r="X118" t="str">
+      <x:c r="AA118" t="str">
         <x:v>Branco</x:v>
       </x:c>
-      <x:c r="Y118" t="str">
+      <x:c r="AB118" t="str">
         <x:v>#FFFFFF</x:v>
       </x:c>
-      <x:c r="Z118" t="str">
+      <x:c r="AC118" t="str">
         <x:v>255,255,255</x:v>
       </x:c>
-      <x:c r="AA118"/>
-      <x:c r="AB118"/>
-      <x:c r="AC118"/>
       <x:c r="AD118" t="str">
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE118" t="str">
-        <x:v>QFC</x:v>
+        <x:v>Potyguar Seridoense</x:v>
       </x:c>
       <x:c r="AF118" t="str">
-        <x:v>Quinho Futebol Clube</x:v>
+        <x:v>Associação Cultural e Desportiva Potyguar Seridoense</x:v>
       </x:c>
     </x:row>
     <x:row r="119">
       <x:c r="A119" t="str">
-        <x:v>RO</x:v>
+        <x:v>RN</x:v>
       </x:c>
       <x:c r="B119" t="str">
-        <x:v>Porto Velho</x:v>
+        <x:v>Parnamirim</x:v>
       </x:c>
       <x:c r="C119"/>
       <x:c r="D119" t="str">
@@ -10407,10 +10407,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G119" t="str">
-        <x:v>Barcelona-RO</x:v>
+        <x:v>QFC</x:v>
       </x:c>
       <x:c r="H119" t="str">
-        <x:v>barcelona_ro.png</x:v>
+        <x:v>qfc.png</x:v>
       </x:c>
       <x:c r="I119" t="str">
         <x:v>PNG</x:v>
@@ -10426,23 +10426,21 @@
       <x:c r="N119" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O119" t="str">
-        <x:v>https://www.footballkitarchive.com/es/campeonato-rondoniense-camisetas-2026-l339/</x:v>
-      </x:c>
+      <x:c r="O119"/>
       <x:c r="P119" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Barcelona-RO%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22QFC%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q119" t="str">
-        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
+        <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R119" t="str">
-        <x:v>Azul / Vermelho</x:v>
+        <x:v>Azul / Branco</x:v>
       </x:c>
       <x:c r="S119" t="str">
-        <x:v>#0057B8 / #D2232A</x:v>
+        <x:v>#0057B8 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T119" t="str">
-        <x:v>0,87,184 / 210,35,42</x:v>
+        <x:v>0,87,184 / 255,255,255</x:v>
       </x:c>
       <x:c r="U119" t="str">
         <x:v>Azul</x:v>
@@ -10454,13 +10452,13 @@
         <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="X119" t="str">
-        <x:v>Vermelho</x:v>
+        <x:v>Branco</x:v>
       </x:c>
       <x:c r="Y119" t="str">
-        <x:v>#D2232A</x:v>
+        <x:v>#FFFFFF</x:v>
       </x:c>
       <x:c r="Z119" t="str">
-        <x:v>210,35,42</x:v>
+        <x:v>255,255,255</x:v>
       </x:c>
       <x:c r="AA119"/>
       <x:c r="AB119"/>
@@ -10469,10 +10467,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE119" t="str">
-        <x:v>Barcelona-RO</x:v>
+        <x:v>QFC</x:v>
       </x:c>
       <x:c r="AF119" t="str">
-        <x:v>Barcelona Futebol Clube</x:v>
+        <x:v>Quinho Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="120">
@@ -10491,10 +10489,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G120" t="str">
-        <x:v>Genus</x:v>
+        <x:v>Barcelona-RO</x:v>
       </x:c>
       <x:c r="H120" t="str">
-        <x:v>genus.png</x:v>
+        <x:v>barcelona_ro.png</x:v>
       </x:c>
       <x:c r="I120" t="str">
         <x:v>PNG</x:v>
@@ -10514,37 +10512,37 @@
         <x:v>https://www.footballkitarchive.com/es/campeonato-rondoniense-camisetas-2026-l339/</x:v>
       </x:c>
       <x:c r="P120" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Genus%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Barcelona-RO%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q120" t="str">
         <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R120" t="str">
-        <x:v>Amarelo / Grená</x:v>
+        <x:v>Azul / Vermelho</x:v>
       </x:c>
       <x:c r="S120" t="str">
-        <x:v>#FFD100 / #7A263A</x:v>
+        <x:v>#0057B8 / #D2232A</x:v>
       </x:c>
       <x:c r="T120" t="str">
-        <x:v>255,209,0 / 122,38,58</x:v>
+        <x:v>0,87,184 / 210,35,42</x:v>
       </x:c>
       <x:c r="U120" t="str">
-        <x:v>Amarelo</x:v>
+        <x:v>Azul</x:v>
       </x:c>
       <x:c r="V120" t="str">
-        <x:v>#FFD100</x:v>
+        <x:v>#0057B8</x:v>
       </x:c>
       <x:c r="W120" t="str">
-        <x:v>255,209,0</x:v>
+        <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="X120" t="str">
-        <x:v>Grená</x:v>
+        <x:v>Vermelho</x:v>
       </x:c>
       <x:c r="Y120" t="str">
-        <x:v>#7A263A</x:v>
+        <x:v>#D2232A</x:v>
       </x:c>
       <x:c r="Z120" t="str">
-        <x:v>122,38,58</x:v>
+        <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="AA120"/>
       <x:c r="AB120"/>
@@ -10553,10 +10551,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE120" t="str">
-        <x:v>Genus</x:v>
+        <x:v>Barcelona-RO</x:v>
       </x:c>
       <x:c r="AF120" t="str">
-        <x:v>Sport Club Genus de Porto Velho</x:v>
+        <x:v>Barcelona Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="121">
@@ -10564,25 +10562,21 @@
         <x:v>RO</x:v>
       </x:c>
       <x:c r="B121" t="str">
-        <x:v>Rolim de Moura</x:v>
-      </x:c>
-      <x:c r="C121" t="str">
-        <x:v>D</x:v>
-      </x:c>
+        <x:v>Porto Velho</x:v>
+      </x:c>
+      <x:c r="C121"/>
       <x:c r="D121" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E121" t="str">
-        <x:v>Uniforme 2026 confirmado: Top Art Uniformes; modelo outro (descrever em obs).</x:v>
-      </x:c>
+      <x:c r="E121"/>
       <x:c r="F121" t="str">
-        <x:v>D</x:v>
+        <x:v>estadual</x:v>
       </x:c>
       <x:c r="G121" t="str">
-        <x:v>Guaporé</x:v>
+        <x:v>Genus</x:v>
       </x:c>
       <x:c r="H121" t="str">
-        <x:v>guapore.png</x:v>
+        <x:v>genus.png</x:v>
       </x:c>
       <x:c r="I121" t="str">
         <x:v>PNG</x:v>
@@ -10602,49 +10596,49 @@
         <x:v>https://www.footballkitarchive.com/es/campeonato-rondoniense-camisetas-2026-l339/</x:v>
       </x:c>
       <x:c r="P121" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Guapor%C3%A9%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Genus%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q121" t="str">
         <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R121" t="str">
-        <x:v>Laranja / Verde</x:v>
+        <x:v>Amarelo / Grená</x:v>
       </x:c>
       <x:c r="S121" t="str">
-        <x:v>#F58220 / #00843D</x:v>
+        <x:v>#FFD100 / #7A263A</x:v>
       </x:c>
       <x:c r="T121" t="str">
-        <x:v>245,130,32 / 0,132,61</x:v>
+        <x:v>255,209,0 / 122,38,58</x:v>
       </x:c>
       <x:c r="U121" t="str">
-        <x:v>Laranja</x:v>
+        <x:v>Amarelo</x:v>
       </x:c>
       <x:c r="V121" t="str">
-        <x:v>#F58220</x:v>
+        <x:v>#FFD100</x:v>
       </x:c>
       <x:c r="W121" t="str">
-        <x:v>245,130,32</x:v>
+        <x:v>255,209,0</x:v>
       </x:c>
       <x:c r="X121" t="str">
-        <x:v>Verde</x:v>
+        <x:v>Grená</x:v>
       </x:c>
       <x:c r="Y121" t="str">
-        <x:v>#00843D</x:v>
+        <x:v>#7A263A</x:v>
       </x:c>
       <x:c r="Z121" t="str">
-        <x:v>0,132,61</x:v>
+        <x:v>122,38,58</x:v>
       </x:c>
       <x:c r="AA121"/>
       <x:c r="AB121"/>
       <x:c r="AC121"/>
       <x:c r="AD121" t="str">
-        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
+        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE121" t="str">
-        <x:v>Guaporé</x:v>
+        <x:v>Genus</x:v>
       </x:c>
       <x:c r="AF121" t="str">
-        <x:v>Guaporé Futebol Clube</x:v>
+        <x:v>Sport Club Genus de Porto Velho</x:v>
       </x:c>
     </x:row>
     <x:row r="122">
@@ -10652,21 +10646,25 @@
         <x:v>RO</x:v>
       </x:c>
       <x:c r="B122" t="str">
-        <x:v>Ji-Paraná</x:v>
-      </x:c>
-      <x:c r="C122"/>
+        <x:v>Rolim de Moura</x:v>
+      </x:c>
+      <x:c r="C122" t="str">
+        <x:v>D</x:v>
+      </x:c>
       <x:c r="D122" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E122"/>
+      <x:c r="E122" t="str">
+        <x:v>Uniforme 2026 confirmado: Top Art Uniformes; modelo outro (descrever em obs).</x:v>
+      </x:c>
       <x:c r="F122" t="str">
-        <x:v>estadual</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="G122" t="str">
-        <x:v>Ji-Paraná</x:v>
+        <x:v>Guaporé</x:v>
       </x:c>
       <x:c r="H122" t="str">
-        <x:v>ji_parana.png</x:v>
+        <x:v>guapore.png</x:v>
       </x:c>
       <x:c r="I122" t="str">
         <x:v>PNG</x:v>
@@ -10683,40 +10681,40 @@
         <x:v>Football Kit Archive</x:v>
       </x:c>
       <x:c r="O122" t="str">
-        <x:v>https://www.footballkitarchive.com/ji-parana-2026-home-kit/453633/</x:v>
+        <x:v>https://www.footballkitarchive.com/es/campeonato-rondoniense-camisetas-2026-l339/</x:v>
       </x:c>
       <x:c r="P122" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Ji-Paran%C3%A1%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Guapor%C3%A9%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q122" t="str">
-        <x:v>REFERÊNCIA 2026 DIRETA</x:v>
+        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R122" t="str">
-        <x:v>Azul / Branco</x:v>
+        <x:v>Laranja / Verde</x:v>
       </x:c>
       <x:c r="S122" t="str">
-        <x:v>#0057B8 / #FFFFFF</x:v>
+        <x:v>#F58220 / #00843D</x:v>
       </x:c>
       <x:c r="T122" t="str">
-        <x:v>0,87,184 / 255,255,255</x:v>
+        <x:v>245,130,32 / 0,132,61</x:v>
       </x:c>
       <x:c r="U122" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Laranja</x:v>
       </x:c>
       <x:c r="V122" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#F58220</x:v>
       </x:c>
       <x:c r="W122" t="str">
-        <x:v>0,87,184</x:v>
+        <x:v>245,130,32</x:v>
       </x:c>
       <x:c r="X122" t="str">
-        <x:v>Branco</x:v>
+        <x:v>Verde</x:v>
       </x:c>
       <x:c r="Y122" t="str">
-        <x:v>#FFFFFF</x:v>
+        <x:v>#00843D</x:v>
       </x:c>
       <x:c r="Z122" t="str">
-        <x:v>255,255,255</x:v>
+        <x:v>0,132,61</x:v>
       </x:c>
       <x:c r="AA122"/>
       <x:c r="AB122"/>
@@ -10725,10 +10723,10 @@
         <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE122" t="str">
-        <x:v>Ji-Paraná</x:v>
+        <x:v>Guaporé</x:v>
       </x:c>
       <x:c r="AF122" t="str">
-        <x:v>Ji-Paraná Futebol Clube</x:v>
+        <x:v>Guaporé Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="123">
@@ -10736,7 +10734,7 @@
         <x:v>RO</x:v>
       </x:c>
       <x:c r="B123" t="str">
-        <x:v>Porto Velho</x:v>
+        <x:v>Ji-Paraná</x:v>
       </x:c>
       <x:c r="C123"/>
       <x:c r="D123" t="str">
@@ -10747,10 +10745,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G123" t="str">
-        <x:v>Rondoniense</x:v>
+        <x:v>Ji-Paraná</x:v>
       </x:c>
       <x:c r="H123" t="str">
-        <x:v>rondoniense.png</x:v>
+        <x:v>ji_parana.png</x:v>
       </x:c>
       <x:c r="I123" t="str">
         <x:v>PNG</x:v>
@@ -10767,22 +10765,22 @@
         <x:v>Football Kit Archive</x:v>
       </x:c>
       <x:c r="O123" t="str">
-        <x:v>https://www.footballkitarchive.com/pt/camisa-titular-rondoniense-2026-448968/</x:v>
+        <x:v>https://www.footballkitarchive.com/ji-parana-2026-home-kit/453633/</x:v>
       </x:c>
       <x:c r="P123" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Rondoniense%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Ji-Paran%C3%A1%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q123" t="str">
         <x:v>REFERÊNCIA 2026 DIRETA</x:v>
       </x:c>
       <x:c r="R123" t="str">
-        <x:v>Azul / Amarelo / Verde</x:v>
+        <x:v>Azul / Branco</x:v>
       </x:c>
       <x:c r="S123" t="str">
-        <x:v>#0057B8 / #FFD100 / #00843D</x:v>
+        <x:v>#0057B8 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T123" t="str">
-        <x:v>0,87,184 / 255,209,0 / 0,132,61</x:v>
+        <x:v>0,87,184 / 255,255,255</x:v>
       </x:c>
       <x:c r="U123" t="str">
         <x:v>Azul</x:v>
@@ -10794,31 +10792,25 @@
         <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="X123" t="str">
-        <x:v>Amarelo</x:v>
+        <x:v>Branco</x:v>
       </x:c>
       <x:c r="Y123" t="str">
-        <x:v>#FFD100</x:v>
+        <x:v>#FFFFFF</x:v>
       </x:c>
       <x:c r="Z123" t="str">
-        <x:v>255,209,0</x:v>
-      </x:c>
-      <x:c r="AA123" t="str">
-        <x:v>Verde</x:v>
-      </x:c>
-      <x:c r="AB123" t="str">
-        <x:v>#00843D</x:v>
-      </x:c>
-      <x:c r="AC123" t="str">
-        <x:v>0,132,61</x:v>
-      </x:c>
+        <x:v>255,255,255</x:v>
+      </x:c>
+      <x:c r="AA123"/>
+      <x:c r="AB123"/>
+      <x:c r="AC123"/>
       <x:c r="AD123" t="str">
         <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE123" t="str">
-        <x:v>Rondoniense</x:v>
+        <x:v>Ji-Paraná</x:v>
       </x:c>
       <x:c r="AF123" t="str">
-        <x:v>Rondoniense Social Clube</x:v>
+        <x:v>Ji-Paraná Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="124">
@@ -10826,7 +10818,7 @@
         <x:v>RO</x:v>
       </x:c>
       <x:c r="B124" t="str">
-        <x:v>Cacoal</x:v>
+        <x:v>Porto Velho</x:v>
       </x:c>
       <x:c r="C124"/>
       <x:c r="D124" t="str">
@@ -10837,10 +10829,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G124" t="str">
-        <x:v>União Cacoalense</x:v>
+        <x:v>Rondoniense</x:v>
       </x:c>
       <x:c r="H124" t="str">
-        <x:v>uniao_cacoalense.png</x:v>
+        <x:v>rondoniense.png</x:v>
       </x:c>
       <x:c r="I124" t="str">
         <x:v>PNG</x:v>
@@ -10857,40 +10849,40 @@
         <x:v>Football Kit Archive</x:v>
       </x:c>
       <x:c r="O124" t="str">
-        <x:v>https://www.footballkitarchive.com/es/camiseta-local-uniao-cacoalense-2026-447072/</x:v>
+        <x:v>https://www.footballkitarchive.com/pt/camisa-titular-rondoniense-2026-448968/</x:v>
       </x:c>
       <x:c r="P124" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Uni%C3%A3o+Cacoalense%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Rondoniense%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q124" t="str">
         <x:v>REFERÊNCIA 2026 DIRETA</x:v>
       </x:c>
       <x:c r="R124" t="str">
-        <x:v>Branco / Azul / Verde</x:v>
+        <x:v>Azul / Amarelo / Verde</x:v>
       </x:c>
       <x:c r="S124" t="str">
-        <x:v>#FFFFFF / #0057B8 / #00843D</x:v>
+        <x:v>#0057B8 / #FFD100 / #00843D</x:v>
       </x:c>
       <x:c r="T124" t="str">
-        <x:v>255,255,255 / 0,87,184 / 0,132,61</x:v>
+        <x:v>0,87,184 / 255,209,0 / 0,132,61</x:v>
       </x:c>
       <x:c r="U124" t="str">
-        <x:v>Branco</x:v>
+        <x:v>Azul</x:v>
       </x:c>
       <x:c r="V124" t="str">
-        <x:v>#FFFFFF</x:v>
+        <x:v>#0057B8</x:v>
       </x:c>
       <x:c r="W124" t="str">
-        <x:v>255,255,255</x:v>
+        <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="X124" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Amarelo</x:v>
       </x:c>
       <x:c r="Y124" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#FFD100</x:v>
       </x:c>
       <x:c r="Z124" t="str">
-        <x:v>0,87,184</x:v>
+        <x:v>255,209,0</x:v>
       </x:c>
       <x:c r="AA124" t="str">
         <x:v>Verde</x:v>
@@ -10905,18 +10897,18 @@
         <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE124" t="str">
-        <x:v>União Cacoalense</x:v>
+        <x:v>Rondoniense</x:v>
       </x:c>
       <x:c r="AF124" t="str">
-        <x:v>Sociedade Esportiva União Cacoalense</x:v>
+        <x:v>Rondoniense Social Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="125">
       <x:c r="A125" t="str">
-        <x:v>RR</x:v>
+        <x:v>RO</x:v>
       </x:c>
       <x:c r="B125" t="str">
-        <x:v>Boa Vista</x:v>
+        <x:v>Cacoal</x:v>
       </x:c>
       <x:c r="C125"/>
       <x:c r="D125" t="str">
@@ -10927,10 +10919,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G125" t="str">
-        <x:v>Atlético Roraima</x:v>
+        <x:v>União Cacoalense</x:v>
       </x:c>
       <x:c r="H125" t="str">
-        <x:v>atletico_roraima.png</x:v>
+        <x:v>uniao_cacoalense.png</x:v>
       </x:c>
       <x:c r="I125" t="str">
         <x:v>PNG</x:v>
@@ -10947,40 +10939,40 @@
         <x:v>Football Kit Archive</x:v>
       </x:c>
       <x:c r="O125" t="str">
-        <x:v>https://www.footballkitarchive.com/pt/campeonato-roraimense-camisas-l1808/</x:v>
+        <x:v>https://www.footballkitarchive.com/es/camiseta-local-uniao-cacoalense-2026-447072/</x:v>
       </x:c>
       <x:c r="P125" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Atl%C3%A9tico+Roraima%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Uni%C3%A3o+Cacoalense%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q125" t="str">
-        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
+        <x:v>REFERÊNCIA 2026 DIRETA</x:v>
       </x:c>
       <x:c r="R125" t="str">
-        <x:v>Grená / Branco / Verde</x:v>
+        <x:v>Branco / Azul / Verde</x:v>
       </x:c>
       <x:c r="S125" t="str">
-        <x:v>#7A263A / #FFFFFF / #00843D</x:v>
+        <x:v>#FFFFFF / #0057B8 / #00843D</x:v>
       </x:c>
       <x:c r="T125" t="str">
-        <x:v>122,38,58 / 255,255,255 / 0,132,61</x:v>
+        <x:v>255,255,255 / 0,87,184 / 0,132,61</x:v>
       </x:c>
       <x:c r="U125" t="str">
-        <x:v>Grená</x:v>
+        <x:v>Branco</x:v>
       </x:c>
       <x:c r="V125" t="str">
-        <x:v>#7A263A</x:v>
+        <x:v>#FFFFFF</x:v>
       </x:c>
       <x:c r="W125" t="str">
-        <x:v>122,38,58</x:v>
+        <x:v>255,255,255</x:v>
       </x:c>
       <x:c r="X125" t="str">
-        <x:v>Branco</x:v>
+        <x:v>Azul</x:v>
       </x:c>
       <x:c r="Y125" t="str">
-        <x:v>#FFFFFF</x:v>
+        <x:v>#0057B8</x:v>
       </x:c>
       <x:c r="Z125" t="str">
-        <x:v>255,255,255</x:v>
+        <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="AA125" t="str">
         <x:v>Verde</x:v>
@@ -10992,13 +10984,13 @@
         <x:v>0,132,61</x:v>
       </x:c>
       <x:c r="AD125" t="str">
-        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE125" t="str">
-        <x:v>Atlético Roraima</x:v>
+        <x:v>União Cacoalense</x:v>
       </x:c>
       <x:c r="AF125" t="str">
-        <x:v>Atlético Roraima Clube</x:v>
+        <x:v>Sociedade Esportiva União Cacoalense</x:v>
       </x:c>
     </x:row>
     <x:row r="126">
@@ -11017,10 +11009,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G126" t="str">
-        <x:v>Baré</x:v>
+        <x:v>Atlético Roraima</x:v>
       </x:c>
       <x:c r="H126" t="str">
-        <x:v>bare.png</x:v>
+        <x:v>atletico_roraima.png</x:v>
       </x:c>
       <x:c r="I126" t="str">
         <x:v>PNG</x:v>
@@ -11036,30 +11028,32 @@
       <x:c r="N126" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O126"/>
+      <x:c r="O126" t="str">
+        <x:v>https://www.footballkitarchive.com/pt/campeonato-roraimense-camisas-l1808/</x:v>
+      </x:c>
       <x:c r="P126" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Bar%C3%A9%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Atl%C3%A9tico+Roraima%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q126" t="str">
-        <x:v>PENDENTE DE FOTO DIRETA</x:v>
+        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R126" t="str">
-        <x:v>Vermelho / Branco</x:v>
+        <x:v>Grená / Branco / Verde</x:v>
       </x:c>
       <x:c r="S126" t="str">
-        <x:v>#D2232A / #FFFFFF</x:v>
+        <x:v>#7A263A / #FFFFFF / #00843D</x:v>
       </x:c>
       <x:c r="T126" t="str">
-        <x:v>210,35,42 / 255,255,255</x:v>
+        <x:v>122,38,58 / 255,255,255 / 0,132,61</x:v>
       </x:c>
       <x:c r="U126" t="str">
-        <x:v>Vermelho</x:v>
+        <x:v>Grená</x:v>
       </x:c>
       <x:c r="V126" t="str">
-        <x:v>#D2232A</x:v>
+        <x:v>#7A263A</x:v>
       </x:c>
       <x:c r="W126" t="str">
-        <x:v>210,35,42</x:v>
+        <x:v>122,38,58</x:v>
       </x:c>
       <x:c r="X126" t="str">
         <x:v>Branco</x:v>
@@ -11070,17 +11064,23 @@
       <x:c r="Z126" t="str">
         <x:v>255,255,255</x:v>
       </x:c>
-      <x:c r="AA126"/>
-      <x:c r="AB126"/>
-      <x:c r="AC126"/>
+      <x:c r="AA126" t="str">
+        <x:v>Verde</x:v>
+      </x:c>
+      <x:c r="AB126" t="str">
+        <x:v>#00843D</x:v>
+      </x:c>
+      <x:c r="AC126" t="str">
+        <x:v>0,132,61</x:v>
+      </x:c>
       <x:c r="AD126" t="str">
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE126" t="str">
-        <x:v>Baré</x:v>
+        <x:v>Atlético Roraima</x:v>
       </x:c>
       <x:c r="AF126" t="str">
-        <x:v>Baré Esporte Clube</x:v>
+        <x:v>Atlético Roraima Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="127">
@@ -11090,23 +11090,19 @@
       <x:c r="B127" t="str">
         <x:v>Boa Vista</x:v>
       </x:c>
-      <x:c r="C127" t="str">
-        <x:v>D</x:v>
-      </x:c>
+      <x:c r="C127"/>
       <x:c r="D127" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E127" t="str">
-        <x:v>Uniforme 2026 confirmado: Tolledo; modelo outro (descrever em obs).</x:v>
-      </x:c>
+      <x:c r="E127"/>
       <x:c r="F127" t="str">
-        <x:v>D</x:v>
+        <x:v>estadual</x:v>
       </x:c>
       <x:c r="G127" t="str">
-        <x:v>Monte Roraima</x:v>
+        <x:v>Baré</x:v>
       </x:c>
       <x:c r="H127" t="str">
-        <x:v>monte_roraima.png</x:v>
+        <x:v>bare.png</x:v>
       </x:c>
       <x:c r="I127" t="str">
         <x:v>PNG</x:v>
@@ -11122,59 +11118,51 @@
       <x:c r="N127" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O127" t="str">
-        <x:v>https://www.footballkitarchive.com/pt/campeonato-roraimense-camisas-l1808/</x:v>
-      </x:c>
+      <x:c r="O127"/>
       <x:c r="P127" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Monte+Roraima%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Bar%C3%A9%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q127" t="str">
-        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
+        <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R127" t="str">
-        <x:v>Ouro / Amarelo / Verde</x:v>
+        <x:v>Vermelho / Branco</x:v>
       </x:c>
       <x:c r="S127" t="str">
-        <x:v>#D4AF37 / #FFD100 / #00843D</x:v>
+        <x:v>#D2232A / #FFFFFF</x:v>
       </x:c>
       <x:c r="T127" t="str">
-        <x:v>212,175,55 / 255,209,0 / 0,132,61</x:v>
+        <x:v>210,35,42 / 255,255,255</x:v>
       </x:c>
       <x:c r="U127" t="str">
-        <x:v>Ouro</x:v>
+        <x:v>Vermelho</x:v>
       </x:c>
       <x:c r="V127" t="str">
-        <x:v>#D4AF37</x:v>
+        <x:v>#D2232A</x:v>
       </x:c>
       <x:c r="W127" t="str">
-        <x:v>212,175,55</x:v>
+        <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="X127" t="str">
-        <x:v>Amarelo</x:v>
+        <x:v>Branco</x:v>
       </x:c>
       <x:c r="Y127" t="str">
-        <x:v>#FFD100</x:v>
+        <x:v>#FFFFFF</x:v>
       </x:c>
       <x:c r="Z127" t="str">
-        <x:v>255,209,0</x:v>
-      </x:c>
-      <x:c r="AA127" t="str">
-        <x:v>Verde</x:v>
-      </x:c>
-      <x:c r="AB127" t="str">
-        <x:v>#00843D</x:v>
-      </x:c>
-      <x:c r="AC127" t="str">
-        <x:v>0,132,61</x:v>
-      </x:c>
+        <x:v>255,255,255</x:v>
+      </x:c>
+      <x:c r="AA127"/>
+      <x:c r="AB127"/>
+      <x:c r="AC127"/>
       <x:c r="AD127" t="str">
-        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
+        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE127" t="str">
-        <x:v>Monte Roraima</x:v>
+        <x:v>Baré</x:v>
       </x:c>
       <x:c r="AF127" t="str">
-        <x:v>Monte Roraima Futebol Clube</x:v>
+        <x:v>Baré Esporte Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="128">
@@ -11184,19 +11172,23 @@
       <x:c r="B128" t="str">
         <x:v>Boa Vista</x:v>
       </x:c>
-      <x:c r="C128"/>
+      <x:c r="C128" t="str">
+        <x:v>D</x:v>
+      </x:c>
       <x:c r="D128" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E128"/>
+      <x:c r="E128" t="str">
+        <x:v>Uniforme 2026 confirmado: Tolledo; modelo outro (descrever em obs).</x:v>
+      </x:c>
       <x:c r="F128" t="str">
-        <x:v>estadual</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="G128" t="str">
-        <x:v>Náutico-RR</x:v>
+        <x:v>Monte Roraima</x:v>
       </x:c>
       <x:c r="H128" t="str">
-        <x:v>nautico_rr.png</x:v>
+        <x:v>monte_roraima.png</x:v>
       </x:c>
       <x:c r="I128" t="str">
         <x:v>PNG</x:v>
@@ -11212,51 +11204,59 @@
       <x:c r="N128" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O128"/>
+      <x:c r="O128" t="str">
+        <x:v>https://www.footballkitarchive.com/pt/campeonato-roraimense-camisas-l1808/</x:v>
+      </x:c>
       <x:c r="P128" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22N%C3%A1utico-RR%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Monte+Roraima%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q128" t="str">
-        <x:v>PENDENTE DE FOTO DIRETA</x:v>
+        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R128" t="str">
-        <x:v>Azul / Branco</x:v>
+        <x:v>Ouro / Amarelo / Verde</x:v>
       </x:c>
       <x:c r="S128" t="str">
-        <x:v>#0057B8 / #FFFFFF</x:v>
+        <x:v>#D4AF37 / #FFD100 / #00843D</x:v>
       </x:c>
       <x:c r="T128" t="str">
-        <x:v>0,87,184 / 255,255,255</x:v>
+        <x:v>212,175,55 / 255,209,0 / 0,132,61</x:v>
       </x:c>
       <x:c r="U128" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Ouro</x:v>
       </x:c>
       <x:c r="V128" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#D4AF37</x:v>
       </x:c>
       <x:c r="W128" t="str">
-        <x:v>0,87,184</x:v>
+        <x:v>212,175,55</x:v>
       </x:c>
       <x:c r="X128" t="str">
-        <x:v>Branco</x:v>
+        <x:v>Amarelo</x:v>
       </x:c>
       <x:c r="Y128" t="str">
-        <x:v>#FFFFFF</x:v>
+        <x:v>#FFD100</x:v>
       </x:c>
       <x:c r="Z128" t="str">
-        <x:v>255,255,255</x:v>
-      </x:c>
-      <x:c r="AA128"/>
-      <x:c r="AB128"/>
-      <x:c r="AC128"/>
+        <x:v>255,209,0</x:v>
+      </x:c>
+      <x:c r="AA128" t="str">
+        <x:v>Verde</x:v>
+      </x:c>
+      <x:c r="AB128" t="str">
+        <x:v>#00843D</x:v>
+      </x:c>
+      <x:c r="AC128" t="str">
+        <x:v>0,132,61</x:v>
+      </x:c>
       <x:c r="AD128" t="str">
-        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE128" t="str">
-        <x:v>Náutico-RR</x:v>
+        <x:v>Monte Roraima</x:v>
       </x:c>
       <x:c r="AF128" t="str">
-        <x:v>Náutico Futebol Clube</x:v>
+        <x:v>Monte Roraima Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="129">
@@ -11264,7 +11264,7 @@
         <x:v>RR</x:v>
       </x:c>
       <x:c r="B129" t="str">
-        <x:v>Mucajaí</x:v>
+        <x:v>Boa Vista</x:v>
       </x:c>
       <x:c r="C129"/>
       <x:c r="D129" t="str">
@@ -11275,10 +11275,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G129" t="str">
-        <x:v>Progresso</x:v>
+        <x:v>Náutico-RR</x:v>
       </x:c>
       <x:c r="H129" t="str">
-        <x:v>progresso.png</x:v>
+        <x:v>nautico_rr.png</x:v>
       </x:c>
       <x:c r="I129" t="str">
         <x:v>PNG</x:v>
@@ -11294,53 +11294,51 @@
       <x:c r="N129" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O129" t="str">
-        <x:v>https://www.footballkitarchive.com/progresso-rr-2026-home-kit-453682/</x:v>
-      </x:c>
+      <x:c r="O129"/>
       <x:c r="P129" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Progresso%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22N%C3%A1utico-RR%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q129" t="str">
-        <x:v>REFERÊNCIA 2026 DIRETA</x:v>
+        <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R129" t="str">
-        <x:v>Verde / Amarelo</x:v>
+        <x:v>Azul / Branco</x:v>
       </x:c>
       <x:c r="S129" t="str">
-        <x:v>#00843D / #FFD100</x:v>
+        <x:v>#0057B8 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T129" t="str">
-        <x:v>0,132,61 / 255,209,0</x:v>
+        <x:v>0,87,184 / 255,255,255</x:v>
       </x:c>
       <x:c r="U129" t="str">
-        <x:v>Verde</x:v>
+        <x:v>Azul</x:v>
       </x:c>
       <x:c r="V129" t="str">
-        <x:v>#00843D</x:v>
+        <x:v>#0057B8</x:v>
       </x:c>
       <x:c r="W129" t="str">
-        <x:v>0,132,61</x:v>
+        <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="X129" t="str">
-        <x:v>Amarelo</x:v>
+        <x:v>Branco</x:v>
       </x:c>
       <x:c r="Y129" t="str">
-        <x:v>#FFD100</x:v>
+        <x:v>#FFFFFF</x:v>
       </x:c>
       <x:c r="Z129" t="str">
-        <x:v>255,209,0</x:v>
+        <x:v>255,255,255</x:v>
       </x:c>
       <x:c r="AA129"/>
       <x:c r="AB129"/>
       <x:c r="AC129"/>
       <x:c r="AD129" t="str">
-        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
+        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE129" t="str">
-        <x:v>Progresso</x:v>
+        <x:v>Náutico-RR</x:v>
       </x:c>
       <x:c r="AF129" t="str">
-        <x:v>Atlético Progresso Clube</x:v>
+        <x:v>Náutico Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="130">
@@ -11348,7 +11346,7 @@
         <x:v>RR</x:v>
       </x:c>
       <x:c r="B130" t="str">
-        <x:v>Boa Vista</x:v>
+        <x:v>Mucajaí</x:v>
       </x:c>
       <x:c r="C130"/>
       <x:c r="D130" t="str">
@@ -11359,10 +11357,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G130" t="str">
-        <x:v>Rio Negro-RR</x:v>
+        <x:v>Progresso</x:v>
       </x:c>
       <x:c r="H130" t="str">
-        <x:v>rio_negro_rr.png</x:v>
+        <x:v>progresso.png</x:v>
       </x:c>
       <x:c r="I130" t="str">
         <x:v>PNG</x:v>
@@ -11378,51 +11376,53 @@
       <x:c r="N130" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O130"/>
+      <x:c r="O130" t="str">
+        <x:v>https://www.footballkitarchive.com/progresso-rr-2026-home-kit-453682/</x:v>
+      </x:c>
       <x:c r="P130" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Rio+Negro-RR%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Progresso%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q130" t="str">
-        <x:v>PENDENTE DE FOTO DIRETA</x:v>
+        <x:v>REFERÊNCIA 2026 DIRETA</x:v>
       </x:c>
       <x:c r="R130" t="str">
-        <x:v>Preto / Branco</x:v>
+        <x:v>Verde / Amarelo</x:v>
       </x:c>
       <x:c r="S130" t="str">
-        <x:v>#000000 / #FFFFFF</x:v>
+        <x:v>#00843D / #FFD100</x:v>
       </x:c>
       <x:c r="T130" t="str">
-        <x:v>0,0,0 / 255,255,255</x:v>
+        <x:v>0,132,61 / 255,209,0</x:v>
       </x:c>
       <x:c r="U130" t="str">
-        <x:v>Preto</x:v>
+        <x:v>Verde</x:v>
       </x:c>
       <x:c r="V130" t="str">
-        <x:v>#000000</x:v>
+        <x:v>#00843D</x:v>
       </x:c>
       <x:c r="W130" t="str">
-        <x:v>0,0,0</x:v>
+        <x:v>0,132,61</x:v>
       </x:c>
       <x:c r="X130" t="str">
-        <x:v>Branco</x:v>
+        <x:v>Amarelo</x:v>
       </x:c>
       <x:c r="Y130" t="str">
-        <x:v>#FFFFFF</x:v>
+        <x:v>#FFD100</x:v>
       </x:c>
       <x:c r="Z130" t="str">
-        <x:v>255,255,255</x:v>
+        <x:v>255,209,0</x:v>
       </x:c>
       <x:c r="AA130"/>
       <x:c r="AB130"/>
       <x:c r="AC130"/>
       <x:c r="AD130" t="str">
-        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE130" t="str">
-        <x:v>Rio Negro-RR</x:v>
+        <x:v>Progresso</x:v>
       </x:c>
       <x:c r="AF130" t="str">
-        <x:v>Atlético Rio Negro Clube</x:v>
+        <x:v>Atlético Progresso Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="131">
@@ -11441,10 +11441,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G131" t="str">
-        <x:v>River-RR</x:v>
+        <x:v>Rio Negro-RR</x:v>
       </x:c>
       <x:c r="H131" t="str">
-        <x:v>river_rr.png</x:v>
+        <x:v>rio_negro_rr.png</x:v>
       </x:c>
       <x:c r="I131" t="str">
         <x:v>PNG</x:v>
@@ -11460,32 +11460,30 @@
       <x:c r="N131" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O131" t="str">
-        <x:v>https://www.footballkitarchive.com/pt/campeonato-roraimense-camisas-l1808/</x:v>
-      </x:c>
+      <x:c r="O131"/>
       <x:c r="P131" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22River-RR%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Rio+Negro-RR%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q131" t="str">
-        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
+        <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R131" t="str">
-        <x:v>Verde / Branco</x:v>
+        <x:v>Preto / Branco</x:v>
       </x:c>
       <x:c r="S131" t="str">
-        <x:v>#00843D / #FFFFFF</x:v>
+        <x:v>#000000 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T131" t="str">
-        <x:v>0,132,61 / 255,255,255</x:v>
+        <x:v>0,0,0 / 255,255,255</x:v>
       </x:c>
       <x:c r="U131" t="str">
-        <x:v>Verde</x:v>
+        <x:v>Preto</x:v>
       </x:c>
       <x:c r="V131" t="str">
-        <x:v>#00843D</x:v>
+        <x:v>#000000</x:v>
       </x:c>
       <x:c r="W131" t="str">
-        <x:v>0,132,61</x:v>
+        <x:v>0,0,0</x:v>
       </x:c>
       <x:c r="X131" t="str">
         <x:v>Branco</x:v>
@@ -11503,10 +11501,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE131" t="str">
-        <x:v>River-RR</x:v>
+        <x:v>Rio Negro-RR</x:v>
       </x:c>
       <x:c r="AF131" t="str">
-        <x:v>River Esporte Clube</x:v>
+        <x:v>Atlético Rio Negro Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="132">
@@ -11516,23 +11514,19 @@
       <x:c r="B132" t="str">
         <x:v>Boa Vista</x:v>
       </x:c>
-      <x:c r="C132" t="str">
-        <x:v>D</x:v>
-      </x:c>
+      <x:c r="C132"/>
       <x:c r="D132" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E132" t="str">
-        <x:v>Uniforme 2026 confirmado: In-House; modelo lisa.</x:v>
-      </x:c>
+      <x:c r="E132"/>
       <x:c r="F132" t="str">
-        <x:v>D</x:v>
+        <x:v>estadual</x:v>
       </x:c>
       <x:c r="G132" t="str">
-        <x:v>São Raimundo-RR</x:v>
+        <x:v>River-RR</x:v>
       </x:c>
       <x:c r="H132" t="str">
-        <x:v>sao_raimundo_rr.png</x:v>
+        <x:v>river_rr.png</x:v>
       </x:c>
       <x:c r="I132" t="str">
         <x:v>PNG</x:v>
@@ -11549,31 +11543,31 @@
         <x:v>Football Kit Archive</x:v>
       </x:c>
       <x:c r="O132" t="str">
-        <x:v>https://www.footballkitarchive.com/sao-raimundo-rr-2026-home-kit-453571/</x:v>
+        <x:v>https://www.footballkitarchive.com/pt/campeonato-roraimense-camisas-l1808/</x:v>
       </x:c>
       <x:c r="P132" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22S%C3%A3o+Raimundo-RR%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22River-RR%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q132" t="str">
-        <x:v>REFERÊNCIA 2026 DIRETA</x:v>
+        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R132" t="str">
-        <x:v>Azul / Branco</x:v>
+        <x:v>Verde / Branco</x:v>
       </x:c>
       <x:c r="S132" t="str">
-        <x:v>#0057B8 / #FFFFFF</x:v>
+        <x:v>#00843D / #FFFFFF</x:v>
       </x:c>
       <x:c r="T132" t="str">
-        <x:v>0,87,184 / 255,255,255</x:v>
+        <x:v>0,132,61 / 255,255,255</x:v>
       </x:c>
       <x:c r="U132" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Verde</x:v>
       </x:c>
       <x:c r="V132" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#00843D</x:v>
       </x:c>
       <x:c r="W132" t="str">
-        <x:v>0,87,184</x:v>
+        <x:v>0,132,61</x:v>
       </x:c>
       <x:c r="X132" t="str">
         <x:v>Branco</x:v>
@@ -11588,35 +11582,39 @@
       <x:c r="AB132"/>
       <x:c r="AC132"/>
       <x:c r="AD132" t="str">
-        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
+        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE132" t="str">
-        <x:v>São Raimundo-RR</x:v>
+        <x:v>River-RR</x:v>
       </x:c>
       <x:c r="AF132" t="str">
-        <x:v>São Raimundo Esporte Clube</x:v>
+        <x:v>River Esporte Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="133">
       <x:c r="A133" t="str">
-        <x:v>RS</x:v>
+        <x:v>RR</x:v>
       </x:c>
       <x:c r="B133" t="str">
-        <x:v>Santa Cruz do Sul</x:v>
-      </x:c>
-      <x:c r="C133"/>
+        <x:v>Boa Vista</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>D</x:v>
+      </x:c>
       <x:c r="D133" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E133"/>
+      <x:c r="E133" t="str">
+        <x:v>Uniforme 2026 confirmado: In-House; modelo lisa.</x:v>
+      </x:c>
       <x:c r="F133" t="str">
-        <x:v>estadual</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="G133" t="str">
-        <x:v>Avenida</x:v>
+        <x:v>São Raimundo-RR</x:v>
       </x:c>
       <x:c r="H133" t="str">
-        <x:v>avenida.png</x:v>
+        <x:v>sao_raimundo_rr.png</x:v>
       </x:c>
       <x:c r="I133" t="str">
         <x:v>PNG</x:v>
@@ -11632,30 +11630,32 @@
       <x:c r="N133" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O133"/>
+      <x:c r="O133" t="str">
+        <x:v>https://www.footballkitarchive.com/sao-raimundo-rr-2026-home-kit-453571/</x:v>
+      </x:c>
       <x:c r="P133" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Avenida%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22S%C3%A3o+Raimundo-RR%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q133" t="str">
-        <x:v>PENDENTE DE FOTO DIRETA</x:v>
+        <x:v>REFERÊNCIA 2026 DIRETA</x:v>
       </x:c>
       <x:c r="R133" t="str">
-        <x:v>Verde / Branco</x:v>
+        <x:v>Azul / Branco</x:v>
       </x:c>
       <x:c r="S133" t="str">
-        <x:v>#00843D / #FFFFFF</x:v>
+        <x:v>#0057B8 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T133" t="str">
-        <x:v>0,132,61 / 255,255,255</x:v>
+        <x:v>0,87,184 / 255,255,255</x:v>
       </x:c>
       <x:c r="U133" t="str">
-        <x:v>Verde</x:v>
+        <x:v>Azul</x:v>
       </x:c>
       <x:c r="V133" t="str">
-        <x:v>#00843D</x:v>
+        <x:v>#0057B8</x:v>
       </x:c>
       <x:c r="W133" t="str">
-        <x:v>0,132,61</x:v>
+        <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="X133" t="str">
         <x:v>Branco</x:v>
@@ -11670,13 +11670,13 @@
       <x:c r="AB133"/>
       <x:c r="AC133"/>
       <x:c r="AD133" t="str">
-        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE133" t="str">
-        <x:v>Avenida</x:v>
+        <x:v>São Raimundo-RR</x:v>
       </x:c>
       <x:c r="AF133" t="str">
-        <x:v>Esporte Clube Avenida</x:v>
+        <x:v>São Raimundo Esporte Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="134">
@@ -11684,7 +11684,7 @@
         <x:v>RS</x:v>
       </x:c>
       <x:c r="B134" t="str">
-        <x:v>Santa Maria</x:v>
+        <x:v>Santa Cruz do Sul</x:v>
       </x:c>
       <x:c r="C134"/>
       <x:c r="D134" t="str">
@@ -11695,10 +11695,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G134" t="str">
-        <x:v>Internacional de Santa Maria</x:v>
+        <x:v>Avenida</x:v>
       </x:c>
       <x:c r="H134" t="str">
-        <x:v>internacional_de_santa_maria.png</x:v>
+        <x:v>avenida.png</x:v>
       </x:c>
       <x:c r="I134" t="str">
         <x:v>PNG</x:v>
@@ -11716,28 +11716,28 @@
       </x:c>
       <x:c r="O134"/>
       <x:c r="P134" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Internacional+de+Santa+Maria%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Avenida%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q134" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R134" t="str">
-        <x:v>Vermelho / Branco</x:v>
+        <x:v>Verde / Branco</x:v>
       </x:c>
       <x:c r="S134" t="str">
-        <x:v>#D2232A / #FFFFFF</x:v>
+        <x:v>#00843D / #FFFFFF</x:v>
       </x:c>
       <x:c r="T134" t="str">
-        <x:v>210,35,42 / 255,255,255</x:v>
+        <x:v>0,132,61 / 255,255,255</x:v>
       </x:c>
       <x:c r="U134" t="str">
-        <x:v>Vermelho</x:v>
+        <x:v>Verde</x:v>
       </x:c>
       <x:c r="V134" t="str">
-        <x:v>#D2232A</x:v>
+        <x:v>#00843D</x:v>
       </x:c>
       <x:c r="W134" t="str">
-        <x:v>210,35,42</x:v>
+        <x:v>0,132,61</x:v>
       </x:c>
       <x:c r="X134" t="str">
         <x:v>Branco</x:v>
@@ -11755,10 +11755,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE134" t="str">
-        <x:v>Internacional de Santa Maria</x:v>
+        <x:v>Avenida</x:v>
       </x:c>
       <x:c r="AF134" t="str">
-        <x:v>Esporte Clube Internacional</x:v>
+        <x:v>Esporte Clube Avenida</x:v>
       </x:c>
     </x:row>
     <x:row r="135">
@@ -11766,7 +11766,7 @@
         <x:v>RS</x:v>
       </x:c>
       <x:c r="B135" t="str">
-        <x:v>Porto Alegre</x:v>
+        <x:v>Santa Maria</x:v>
       </x:c>
       <x:c r="C135"/>
       <x:c r="D135" t="str">
@@ -11777,10 +11777,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G135" t="str">
-        <x:v>Monsoon</x:v>
+        <x:v>Internacional de Santa Maria</x:v>
       </x:c>
       <x:c r="H135" t="str">
-        <x:v>monsoon.png</x:v>
+        <x:v>internacional_de_santa_maria.png</x:v>
       </x:c>
       <x:c r="I135" t="str">
         <x:v>PNG</x:v>
@@ -11798,28 +11798,28 @@
       </x:c>
       <x:c r="O135"/>
       <x:c r="P135" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Monsoon%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Internacional+de+Santa+Maria%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q135" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R135" t="str">
-        <x:v>Azul / Branco</x:v>
+        <x:v>Vermelho / Branco</x:v>
       </x:c>
       <x:c r="S135" t="str">
-        <x:v>#0057B8 / #FFFFFF</x:v>
+        <x:v>#D2232A / #FFFFFF</x:v>
       </x:c>
       <x:c r="T135" t="str">
-        <x:v>0,87,184 / 255,255,255</x:v>
+        <x:v>210,35,42 / 255,255,255</x:v>
       </x:c>
       <x:c r="U135" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Vermelho</x:v>
       </x:c>
       <x:c r="V135" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#D2232A</x:v>
       </x:c>
       <x:c r="W135" t="str">
-        <x:v>0,87,184</x:v>
+        <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="X135" t="str">
         <x:v>Branco</x:v>
@@ -11837,10 +11837,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE135" t="str">
-        <x:v>Monsoon</x:v>
+        <x:v>Internacional de Santa Maria</x:v>
       </x:c>
       <x:c r="AF135" t="str">
-        <x:v>Monsoon Futebol Clube</x:v>
+        <x:v>Esporte Clube Internacional</x:v>
       </x:c>
     </x:row>
     <x:row r="136">
@@ -11848,7 +11848,7 @@
         <x:v>RS</x:v>
       </x:c>
       <x:c r="B136" t="str">
-        <x:v>Novo Hamburgo</x:v>
+        <x:v>Porto Alegre</x:v>
       </x:c>
       <x:c r="C136"/>
       <x:c r="D136" t="str">
@@ -11859,10 +11859,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G136" t="str">
-        <x:v>Novo Hamburgo</x:v>
+        <x:v>Monsoon</x:v>
       </x:c>
       <x:c r="H136" t="str">
-        <x:v>novo_hamburgo.png</x:v>
+        <x:v>monsoon.png</x:v>
       </x:c>
       <x:c r="I136" t="str">
         <x:v>PNG</x:v>
@@ -11880,7 +11880,7 @@
       </x:c>
       <x:c r="O136"/>
       <x:c r="P136" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Novo+Hamburgo%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Monsoon%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q136" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
@@ -11919,36 +11919,32 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE136" t="str">
-        <x:v>Novo Hamburgo</x:v>
+        <x:v>Monsoon</x:v>
       </x:c>
       <x:c r="AF136" t="str">
-        <x:v>Esporte Clube Novo Hamburgo</x:v>
+        <x:v>Monsoon Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="137">
       <x:c r="A137" t="str">
-        <x:v>SC</x:v>
+        <x:v>RS</x:v>
       </x:c>
       <x:c r="B137" t="str">
-        <x:v>Blumenau</x:v>
-      </x:c>
-      <x:c r="C137" t="str">
-        <x:v>D</x:v>
-      </x:c>
+        <x:v>Novo Hamburgo</x:v>
+      </x:c>
+      <x:c r="C137"/>
       <x:c r="D137" t="str">
-        <x:v>não</x:v>
-      </x:c>
-      <x:c r="E137" t="str">
-        <x:v>Uniforme 2026 confirmado: Finta; modelo faixa horizontal.</x:v>
-      </x:c>
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="E137"/>
       <x:c r="F137" t="str">
-        <x:v>D</x:v>
+        <x:v>estadual</x:v>
       </x:c>
       <x:c r="G137" t="str">
-        <x:v>Blumenau</x:v>
+        <x:v>Novo Hamburgo</x:v>
       </x:c>
       <x:c r="H137" t="str">
-        <x:v>blumenau.png</x:v>
+        <x:v>novo_hamburgo.png</x:v>
       </x:c>
       <x:c r="I137" t="str">
         <x:v>PNG</x:v>
@@ -11966,55 +11962,49 @@
       </x:c>
       <x:c r="O137"/>
       <x:c r="P137" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Blumenau%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Novo+Hamburgo%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q137" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R137" t="str">
-        <x:v>Branco / Grená / Verde</x:v>
+        <x:v>Azul / Branco</x:v>
       </x:c>
       <x:c r="S137" t="str">
-        <x:v>#FFFFFF / #7A263A / #00843D</x:v>
+        <x:v>#0057B8 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T137" t="str">
-        <x:v>255,255,255 / 122,38,58 / 0,132,61</x:v>
+        <x:v>0,87,184 / 255,255,255</x:v>
       </x:c>
       <x:c r="U137" t="str">
+        <x:v>Azul</x:v>
+      </x:c>
+      <x:c r="V137" t="str">
+        <x:v>#0057B8</x:v>
+      </x:c>
+      <x:c r="W137" t="str">
+        <x:v>0,87,184</x:v>
+      </x:c>
+      <x:c r="X137" t="str">
         <x:v>Branco</x:v>
       </x:c>
-      <x:c r="V137" t="str">
+      <x:c r="Y137" t="str">
         <x:v>#FFFFFF</x:v>
       </x:c>
-      <x:c r="W137" t="str">
+      <x:c r="Z137" t="str">
         <x:v>255,255,255</x:v>
       </x:c>
-      <x:c r="X137" t="str">
-        <x:v>Grená</x:v>
-      </x:c>
-      <x:c r="Y137" t="str">
-        <x:v>#7A263A</x:v>
-      </x:c>
-      <x:c r="Z137" t="str">
-        <x:v>122,38,58</x:v>
-      </x:c>
-      <x:c r="AA137" t="str">
-        <x:v>Verde</x:v>
-      </x:c>
-      <x:c r="AB137" t="str">
-        <x:v>#00843D</x:v>
-      </x:c>
-      <x:c r="AC137" t="str">
-        <x:v>0,132,61</x:v>
-      </x:c>
+      <x:c r="AA137"/>
+      <x:c r="AB137"/>
+      <x:c r="AC137"/>
       <x:c r="AD137" t="str">
-        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
+        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE137" t="str">
-        <x:v>Blumenau</x:v>
+        <x:v>Novo Hamburgo</x:v>
       </x:c>
       <x:c r="AF137" t="str">
-        <x:v>Blumenau Esporte Clube SAF</x:v>
+        <x:v>Esporte Clube Novo Hamburgo</x:v>
       </x:c>
     </x:row>
     <x:row r="138">
@@ -12022,21 +12012,25 @@
         <x:v>SC</x:v>
       </x:c>
       <x:c r="B138" t="str">
-        <x:v>Camboriú</x:v>
-      </x:c>
-      <x:c r="C138"/>
+        <x:v>Blumenau</x:v>
+      </x:c>
+      <x:c r="C138" t="str">
+        <x:v>D</x:v>
+      </x:c>
       <x:c r="D138" t="str">
-        <x:v>sim</x:v>
-      </x:c>
-      <x:c r="E138"/>
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="E138" t="str">
+        <x:v>Uniforme 2026 confirmado: Finta; modelo faixa horizontal.</x:v>
+      </x:c>
       <x:c r="F138" t="str">
-        <x:v>estadual</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="G138" t="str">
-        <x:v>Camboriú</x:v>
+        <x:v>Blumenau</x:v>
       </x:c>
       <x:c r="H138" t="str">
-        <x:v>camboriu.png</x:v>
+        <x:v>blumenau.png</x:v>
       </x:c>
       <x:c r="I138" t="str">
         <x:v>PNG</x:v>
@@ -12054,49 +12048,55 @@
       </x:c>
       <x:c r="O138"/>
       <x:c r="P138" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Cambori%C3%BA%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Blumenau%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q138" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R138" t="str">
-        <x:v>Verde / Branco</x:v>
+        <x:v>Branco / Grená / Verde</x:v>
       </x:c>
       <x:c r="S138" t="str">
-        <x:v>#00843D / #FFFFFF</x:v>
+        <x:v>#FFFFFF / #7A263A / #00843D</x:v>
       </x:c>
       <x:c r="T138" t="str">
-        <x:v>0,132,61 / 255,255,255</x:v>
+        <x:v>255,255,255 / 122,38,58 / 0,132,61</x:v>
       </x:c>
       <x:c r="U138" t="str">
+        <x:v>Branco</x:v>
+      </x:c>
+      <x:c r="V138" t="str">
+        <x:v>#FFFFFF</x:v>
+      </x:c>
+      <x:c r="W138" t="str">
+        <x:v>255,255,255</x:v>
+      </x:c>
+      <x:c r="X138" t="str">
+        <x:v>Grená</x:v>
+      </x:c>
+      <x:c r="Y138" t="str">
+        <x:v>#7A263A</x:v>
+      </x:c>
+      <x:c r="Z138" t="str">
+        <x:v>122,38,58</x:v>
+      </x:c>
+      <x:c r="AA138" t="str">
         <x:v>Verde</x:v>
       </x:c>
-      <x:c r="V138" t="str">
+      <x:c r="AB138" t="str">
         <x:v>#00843D</x:v>
       </x:c>
-      <x:c r="W138" t="str">
+      <x:c r="AC138" t="str">
         <x:v>0,132,61</x:v>
       </x:c>
-      <x:c r="X138" t="str">
-        <x:v>Branco</x:v>
-      </x:c>
-      <x:c r="Y138" t="str">
-        <x:v>#FFFFFF</x:v>
-      </x:c>
-      <x:c r="Z138" t="str">
-        <x:v>255,255,255</x:v>
-      </x:c>
-      <x:c r="AA138"/>
-      <x:c r="AB138"/>
-      <x:c r="AC138"/>
       <x:c r="AD138" t="str">
-        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE138" t="str">
-        <x:v>Camboriú</x:v>
+        <x:v>Blumenau</x:v>
       </x:c>
       <x:c r="AF138" t="str">
-        <x:v>Camboriú Futebol Clube</x:v>
+        <x:v>Blumenau Esporte Clube SAF</x:v>
       </x:c>
     </x:row>
     <x:row r="139">
@@ -12104,7 +12104,7 @@
         <x:v>SC</x:v>
       </x:c>
       <x:c r="B139" t="str">
-        <x:v>Brusque</x:v>
+        <x:v>Camboriú</x:v>
       </x:c>
       <x:c r="C139"/>
       <x:c r="D139" t="str">
@@ -12115,10 +12115,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G139" t="str">
-        <x:v>Carlos Renaux</x:v>
+        <x:v>Camboriú</x:v>
       </x:c>
       <x:c r="H139" t="str">
-        <x:v>carlos_renaux.png</x:v>
+        <x:v>camboriu.png</x:v>
       </x:c>
       <x:c r="I139" t="str">
         <x:v>PNG</x:v>
@@ -12136,55 +12136,49 @@
       </x:c>
       <x:c r="O139"/>
       <x:c r="P139" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Carlos+Renaux%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Cambori%C3%BA%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q139" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R139" t="str">
-        <x:v>Vermelho / Azul / Branco</x:v>
+        <x:v>Verde / Branco</x:v>
       </x:c>
       <x:c r="S139" t="str">
-        <x:v>#D2232A / #0057B8 / #FFFFFF</x:v>
+        <x:v>#00843D / #FFFFFF</x:v>
       </x:c>
       <x:c r="T139" t="str">
-        <x:v>210,35,42 / 0,87,184 / 255,255,255</x:v>
+        <x:v>0,132,61 / 255,255,255</x:v>
       </x:c>
       <x:c r="U139" t="str">
-        <x:v>Vermelho</x:v>
+        <x:v>Verde</x:v>
       </x:c>
       <x:c r="V139" t="str">
-        <x:v>#D2232A</x:v>
+        <x:v>#00843D</x:v>
       </x:c>
       <x:c r="W139" t="str">
-        <x:v>210,35,42</x:v>
+        <x:v>0,132,61</x:v>
       </x:c>
       <x:c r="X139" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Branco</x:v>
       </x:c>
       <x:c r="Y139" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#FFFFFF</x:v>
       </x:c>
       <x:c r="Z139" t="str">
-        <x:v>0,87,184</x:v>
-      </x:c>
-      <x:c r="AA139" t="str">
-        <x:v>Branco</x:v>
-      </x:c>
-      <x:c r="AB139" t="str">
-        <x:v>#FFFFFF</x:v>
-      </x:c>
-      <x:c r="AC139" t="str">
         <x:v>255,255,255</x:v>
       </x:c>
+      <x:c r="AA139"/>
+      <x:c r="AB139"/>
+      <x:c r="AC139"/>
       <x:c r="AD139" t="str">
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE139" t="str">
-        <x:v>Carlos Renaux</x:v>
+        <x:v>Camboriú</x:v>
       </x:c>
       <x:c r="AF139" t="str">
-        <x:v>Clube Atlético Carlos Renaux</x:v>
+        <x:v>Camboriú Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="140">
@@ -12192,7 +12186,7 @@
         <x:v>SC</x:v>
       </x:c>
       <x:c r="B140" t="str">
-        <x:v>Concórdia</x:v>
+        <x:v>Brusque</x:v>
       </x:c>
       <x:c r="C140"/>
       <x:c r="D140" t="str">
@@ -12203,10 +12197,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G140" t="str">
-        <x:v>Concórdia</x:v>
+        <x:v>Carlos Renaux</x:v>
       </x:c>
       <x:c r="H140" t="str">
-        <x:v>concordia.png</x:v>
+        <x:v>carlos_renaux.png</x:v>
       </x:c>
       <x:c r="I140" t="str">
         <x:v>PNG</x:v>
@@ -12224,19 +12218,19 @@
       </x:c>
       <x:c r="O140"/>
       <x:c r="P140" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Conc%C3%B3rdia%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Carlos+Renaux%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q140" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R140" t="str">
-        <x:v>Vermelho / Branco</x:v>
+        <x:v>Vermelho / Azul / Branco</x:v>
       </x:c>
       <x:c r="S140" t="str">
-        <x:v>#D2232A / #FFFFFF</x:v>
+        <x:v>#D2232A / #0057B8 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T140" t="str">
-        <x:v>210,35,42 / 255,255,255</x:v>
+        <x:v>210,35,42 / 0,87,184 / 255,255,255</x:v>
       </x:c>
       <x:c r="U140" t="str">
         <x:v>Vermelho</x:v>
@@ -12248,25 +12242,31 @@
         <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="X140" t="str">
+        <x:v>Azul</x:v>
+      </x:c>
+      <x:c r="Y140" t="str">
+        <x:v>#0057B8</x:v>
+      </x:c>
+      <x:c r="Z140" t="str">
+        <x:v>0,87,184</x:v>
+      </x:c>
+      <x:c r="AA140" t="str">
         <x:v>Branco</x:v>
       </x:c>
-      <x:c r="Y140" t="str">
+      <x:c r="AB140" t="str">
         <x:v>#FFFFFF</x:v>
       </x:c>
-      <x:c r="Z140" t="str">
+      <x:c r="AC140" t="str">
         <x:v>255,255,255</x:v>
       </x:c>
-      <x:c r="AA140"/>
-      <x:c r="AB140"/>
-      <x:c r="AC140"/>
       <x:c r="AD140" t="str">
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE140" t="str">
-        <x:v>Concórdia</x:v>
+        <x:v>Carlos Renaux</x:v>
       </x:c>
       <x:c r="AF140" t="str">
-        <x:v>Concórdia Atlético Clube</x:v>
+        <x:v>Clube Atlético Carlos Renaux</x:v>
       </x:c>
     </x:row>
     <x:row r="141">
@@ -12274,25 +12274,21 @@
         <x:v>SC</x:v>
       </x:c>
       <x:c r="B141" t="str">
-        <x:v>Rio do Sul</x:v>
-      </x:c>
-      <x:c r="C141" t="str">
-        <x:v>D</x:v>
-      </x:c>
+        <x:v>Concórdia</x:v>
+      </x:c>
+      <x:c r="C141"/>
       <x:c r="D141" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E141" t="str">
-        <x:v>Uniforme 2026 confirmado: Athleta; modelo lisa.</x:v>
-      </x:c>
+      <x:c r="E141"/>
       <x:c r="F141" t="str">
-        <x:v>D</x:v>
+        <x:v>estadual</x:v>
       </x:c>
       <x:c r="G141" t="str">
-        <x:v>Santa Catarina</x:v>
+        <x:v>Concórdia</x:v>
       </x:c>
       <x:c r="H141" t="str">
-        <x:v>santa_catarina.png</x:v>
+        <x:v>concordia.png</x:v>
       </x:c>
       <x:c r="I141" t="str">
         <x:v>PNG</x:v>
@@ -12310,71 +12306,75 @@
       </x:c>
       <x:c r="O141"/>
       <x:c r="P141" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Santa+Catarina%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Conc%C3%B3rdia%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q141" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R141" t="str">
-        <x:v>Laranja / Preto</x:v>
+        <x:v>Vermelho / Branco</x:v>
       </x:c>
       <x:c r="S141" t="str">
-        <x:v>#F58220 / #000000</x:v>
+        <x:v>#D2232A / #FFFFFF</x:v>
       </x:c>
       <x:c r="T141" t="str">
-        <x:v>245,130,32 / 0,0,0</x:v>
+        <x:v>210,35,42 / 255,255,255</x:v>
       </x:c>
       <x:c r="U141" t="str">
-        <x:v>Laranja</x:v>
+        <x:v>Vermelho</x:v>
       </x:c>
       <x:c r="V141" t="str">
-        <x:v>#F58220</x:v>
+        <x:v>#D2232A</x:v>
       </x:c>
       <x:c r="W141" t="str">
-        <x:v>245,130,32</x:v>
+        <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="X141" t="str">
-        <x:v>Preto</x:v>
+        <x:v>Branco</x:v>
       </x:c>
       <x:c r="Y141" t="str">
-        <x:v>#000000</x:v>
+        <x:v>#FFFFFF</x:v>
       </x:c>
       <x:c r="Z141" t="str">
-        <x:v>0,0,0</x:v>
+        <x:v>255,255,255</x:v>
       </x:c>
       <x:c r="AA141"/>
       <x:c r="AB141"/>
       <x:c r="AC141"/>
       <x:c r="AD141" t="str">
-        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
+        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE141" t="str">
-        <x:v>Santa Catarina</x:v>
+        <x:v>Concórdia</x:v>
       </x:c>
       <x:c r="AF141" t="str">
-        <x:v>Santa Catarina Clube</x:v>
+        <x:v>Concórdia Atlético Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" t="str">
-        <x:v>SE</x:v>
+        <x:v>SC</x:v>
       </x:c>
       <x:c r="B142" t="str">
-        <x:v>Propriá</x:v>
-      </x:c>
-      <x:c r="C142"/>
+        <x:v>Rio do Sul</x:v>
+      </x:c>
+      <x:c r="C142" t="str">
+        <x:v>D</x:v>
+      </x:c>
       <x:c r="D142" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E142"/>
+      <x:c r="E142" t="str">
+        <x:v>Uniforme 2026 confirmado: Athleta; modelo lisa.</x:v>
+      </x:c>
       <x:c r="F142" t="str">
-        <x:v>estadual</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="G142" t="str">
-        <x:v>América de Propriá</x:v>
+        <x:v>Santa Catarina</x:v>
       </x:c>
       <x:c r="H142" t="str">
-        <x:v>america_de_propria.png</x:v>
+        <x:v>santa_catarina.png</x:v>
       </x:c>
       <x:c r="I142" t="str">
         <x:v>PNG</x:v>
@@ -12390,53 +12390,51 @@
       <x:c r="N142" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O142" t="str">
-        <x:v>https://www.footballkitarchive.com/pt/campeonato-sergipano-kits/</x:v>
-      </x:c>
+      <x:c r="O142"/>
       <x:c r="P142" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Am%C3%A9rica+de+Propri%C3%A1%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Santa+Catarina%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q142" t="str">
-        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
+        <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R142" t="str">
-        <x:v>Vermelho / Branco</x:v>
+        <x:v>Laranja / Preto</x:v>
       </x:c>
       <x:c r="S142" t="str">
-        <x:v>#D2232A / #FFFFFF</x:v>
+        <x:v>#F58220 / #000000</x:v>
       </x:c>
       <x:c r="T142" t="str">
-        <x:v>210,35,42 / 255,255,255</x:v>
+        <x:v>245,130,32 / 0,0,0</x:v>
       </x:c>
       <x:c r="U142" t="str">
-        <x:v>Vermelho</x:v>
+        <x:v>Laranja</x:v>
       </x:c>
       <x:c r="V142" t="str">
-        <x:v>#D2232A</x:v>
+        <x:v>#F58220</x:v>
       </x:c>
       <x:c r="W142" t="str">
-        <x:v>210,35,42</x:v>
+        <x:v>245,130,32</x:v>
       </x:c>
       <x:c r="X142" t="str">
-        <x:v>Branco</x:v>
+        <x:v>Preto</x:v>
       </x:c>
       <x:c r="Y142" t="str">
-        <x:v>#FFFFFF</x:v>
+        <x:v>#000000</x:v>
       </x:c>
       <x:c r="Z142" t="str">
-        <x:v>255,255,255</x:v>
+        <x:v>0,0,0</x:v>
       </x:c>
       <x:c r="AA142"/>
       <x:c r="AB142"/>
       <x:c r="AC142"/>
       <x:c r="AD142" t="str">
-        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE142" t="str">
-        <x:v>América de Propriá</x:v>
+        <x:v>Santa Catarina</x:v>
       </x:c>
       <x:c r="AF142" t="str">
-        <x:v>América Futebol Clube</x:v>
+        <x:v>Santa Catarina Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="143">
@@ -12444,7 +12442,7 @@
         <x:v>SE</x:v>
       </x:c>
       <x:c r="B143" t="str">
-        <x:v>Nossa Senhora da Glória</x:v>
+        <x:v>Propriá</x:v>
       </x:c>
       <x:c r="C143"/>
       <x:c r="D143" t="str">
@@ -12455,10 +12453,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G143" t="str">
-        <x:v>Atlético Gloriense</x:v>
+        <x:v>América de Propriá</x:v>
       </x:c>
       <x:c r="H143" t="str">
-        <x:v>atletico_gloriense.png</x:v>
+        <x:v>america_de_propria.png</x:v>
       </x:c>
       <x:c r="I143" t="str">
         <x:v>PNG</x:v>
@@ -12478,7 +12476,7 @@
         <x:v>https://www.footballkitarchive.com/pt/campeonato-sergipano-kits/</x:v>
       </x:c>
       <x:c r="P143" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Atl%C3%A9tico+Gloriense%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Am%C3%A9rica+de+Propri%C3%A1%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q143" t="str">
         <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
@@ -12517,10 +12515,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE143" t="str">
-        <x:v>Atlético Gloriense</x:v>
+        <x:v>América de Propriá</x:v>
       </x:c>
       <x:c r="AF143" t="str">
-        <x:v>Associação Desportiva Atlético Gloriense</x:v>
+        <x:v>América Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
@@ -12528,7 +12526,7 @@
         <x:v>SE</x:v>
       </x:c>
       <x:c r="B144" t="str">
-        <x:v>Aracaju</x:v>
+        <x:v>Nossa Senhora da Glória</x:v>
       </x:c>
       <x:c r="C144"/>
       <x:c r="D144" t="str">
@@ -12539,10 +12537,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G144" t="str">
-        <x:v>Desportiva Aracaju</x:v>
+        <x:v>Atlético Gloriense</x:v>
       </x:c>
       <x:c r="H144" t="str">
-        <x:v>desportiva_aracaju.png</x:v>
+        <x:v>atletico_gloriense.png</x:v>
       </x:c>
       <x:c r="I144" t="str">
         <x:v>PNG</x:v>
@@ -12562,28 +12560,28 @@
         <x:v>https://www.footballkitarchive.com/pt/campeonato-sergipano-kits/</x:v>
       </x:c>
       <x:c r="P144" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Desportiva+Aracaju%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Atl%C3%A9tico+Gloriense%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q144" t="str">
         <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R144" t="str">
-        <x:v>Azul / Branco</x:v>
+        <x:v>Vermelho / Branco</x:v>
       </x:c>
       <x:c r="S144" t="str">
-        <x:v>#0057B8 / #FFFFFF</x:v>
+        <x:v>#D2232A / #FFFFFF</x:v>
       </x:c>
       <x:c r="T144" t="str">
-        <x:v>0,87,184 / 255,255,255</x:v>
+        <x:v>210,35,42 / 255,255,255</x:v>
       </x:c>
       <x:c r="U144" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Vermelho</x:v>
       </x:c>
       <x:c r="V144" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#D2232A</x:v>
       </x:c>
       <x:c r="W144" t="str">
-        <x:v>0,87,184</x:v>
+        <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="X144" t="str">
         <x:v>Branco</x:v>
@@ -12601,10 +12599,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE144" t="str">
-        <x:v>Desportiva Aracaju</x:v>
+        <x:v>Atlético Gloriense</x:v>
       </x:c>
       <x:c r="AF144" t="str">
-        <x:v>Associação Desportiva Aracaju</x:v>
+        <x:v>Associação Desportiva Atlético Gloriense</x:v>
       </x:c>
     </x:row>
     <x:row r="145">
@@ -12612,7 +12610,7 @@
         <x:v>SE</x:v>
       </x:c>
       <x:c r="B145" t="str">
-        <x:v>Nossa Senhora das Dores</x:v>
+        <x:v>Aracaju</x:v>
       </x:c>
       <x:c r="C145"/>
       <x:c r="D145" t="str">
@@ -12623,10 +12621,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G145" t="str">
-        <x:v>Dorense</x:v>
+        <x:v>Desportiva Aracaju</x:v>
       </x:c>
       <x:c r="H145" t="str">
-        <x:v>dorense.png</x:v>
+        <x:v>desportiva_aracaju.png</x:v>
       </x:c>
       <x:c r="I145" t="str">
         <x:v>PNG</x:v>
@@ -12646,28 +12644,28 @@
         <x:v>https://www.footballkitarchive.com/pt/campeonato-sergipano-kits/</x:v>
       </x:c>
       <x:c r="P145" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Dorense%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Desportiva+Aracaju%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q145" t="str">
         <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R145" t="str">
-        <x:v>Verde / Branco</x:v>
+        <x:v>Azul / Branco</x:v>
       </x:c>
       <x:c r="S145" t="str">
-        <x:v>#00843D / #FFFFFF</x:v>
+        <x:v>#0057B8 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T145" t="str">
-        <x:v>0,132,61 / 255,255,255</x:v>
+        <x:v>0,87,184 / 255,255,255</x:v>
       </x:c>
       <x:c r="U145" t="str">
-        <x:v>Verde</x:v>
+        <x:v>Azul</x:v>
       </x:c>
       <x:c r="V145" t="str">
-        <x:v>#00843D</x:v>
+        <x:v>#0057B8</x:v>
       </x:c>
       <x:c r="W145" t="str">
-        <x:v>0,132,61</x:v>
+        <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="X145" t="str">
         <x:v>Branco</x:v>
@@ -12685,10 +12683,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE145" t="str">
-        <x:v>Dorense</x:v>
+        <x:v>Desportiva Aracaju</x:v>
       </x:c>
       <x:c r="AF145" t="str">
-        <x:v>Dorense Futebol Clube</x:v>
+        <x:v>Associação Desportiva Aracaju</x:v>
       </x:c>
     </x:row>
     <x:row r="146">
@@ -12696,7 +12694,7 @@
         <x:v>SE</x:v>
       </x:c>
       <x:c r="B146" t="str">
-        <x:v>Barra dos Coqueiros</x:v>
+        <x:v>Nossa Senhora das Dores</x:v>
       </x:c>
       <x:c r="C146"/>
       <x:c r="D146" t="str">
@@ -12707,10 +12705,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G146" t="str">
-        <x:v>Falcon</x:v>
+        <x:v>Dorense</x:v>
       </x:c>
       <x:c r="H146" t="str">
-        <x:v>falcon.png</x:v>
+        <x:v>dorense.png</x:v>
       </x:c>
       <x:c r="I146" t="str">
         <x:v>PNG</x:v>
@@ -12730,28 +12728,28 @@
         <x:v>https://www.footballkitarchive.com/pt/campeonato-sergipano-kits/</x:v>
       </x:c>
       <x:c r="P146" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Falcon%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Dorense%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q146" t="str">
         <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R146" t="str">
-        <x:v>Roxo / Branco</x:v>
+        <x:v>Verde / Branco</x:v>
       </x:c>
       <x:c r="S146" t="str">
-        <x:v>#6F2C91 / #FFFFFF</x:v>
+        <x:v>#00843D / #FFFFFF</x:v>
       </x:c>
       <x:c r="T146" t="str">
-        <x:v>111,44,145 / 255,255,255</x:v>
+        <x:v>0,132,61 / 255,255,255</x:v>
       </x:c>
       <x:c r="U146" t="str">
-        <x:v>Roxo</x:v>
+        <x:v>Verde</x:v>
       </x:c>
       <x:c r="V146" t="str">
-        <x:v>#6F2C91</x:v>
+        <x:v>#00843D</x:v>
       </x:c>
       <x:c r="W146" t="str">
-        <x:v>111,44,145</x:v>
+        <x:v>0,132,61</x:v>
       </x:c>
       <x:c r="X146" t="str">
         <x:v>Branco</x:v>
@@ -12769,10 +12767,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE146" t="str">
-        <x:v>Falcon</x:v>
+        <x:v>Dorense</x:v>
       </x:c>
       <x:c r="AF146" t="str">
-        <x:v>Falcon Futebol Clube</x:v>
+        <x:v>Dorense Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="147">
@@ -12780,7 +12778,7 @@
         <x:v>SE</x:v>
       </x:c>
       <x:c r="B147" t="str">
-        <x:v>Porto da Folha</x:v>
+        <x:v>Barra dos Coqueiros</x:v>
       </x:c>
       <x:c r="C147"/>
       <x:c r="D147" t="str">
@@ -12791,10 +12789,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G147" t="str">
-        <x:v>Guarany de Porto da Folha</x:v>
+        <x:v>Falcon</x:v>
       </x:c>
       <x:c r="H147" t="str">
-        <x:v>guarany_de_porto_da_folha.png</x:v>
+        <x:v>falcon.png</x:v>
       </x:c>
       <x:c r="I147" t="str">
         <x:v>PNG</x:v>
@@ -12814,28 +12812,28 @@
         <x:v>https://www.footballkitarchive.com/pt/campeonato-sergipano-kits/</x:v>
       </x:c>
       <x:c r="P147" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Guarany+de+Porto+da+Folha%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Falcon%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q147" t="str">
         <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R147" t="str">
-        <x:v>Vermelho / Branco</x:v>
+        <x:v>Roxo / Branco</x:v>
       </x:c>
       <x:c r="S147" t="str">
-        <x:v>#D2232A / #FFFFFF</x:v>
+        <x:v>#6F2C91 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T147" t="str">
-        <x:v>210,35,42 / 255,255,255</x:v>
+        <x:v>111,44,145 / 255,255,255</x:v>
       </x:c>
       <x:c r="U147" t="str">
-        <x:v>Vermelho</x:v>
+        <x:v>Roxo</x:v>
       </x:c>
       <x:c r="V147" t="str">
-        <x:v>#D2232A</x:v>
+        <x:v>#6F2C91</x:v>
       </x:c>
       <x:c r="W147" t="str">
-        <x:v>210,35,42</x:v>
+        <x:v>111,44,145</x:v>
       </x:c>
       <x:c r="X147" t="str">
         <x:v>Branco</x:v>
@@ -12853,18 +12851,18 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE147" t="str">
-        <x:v>Guarany de Porto da Folha</x:v>
+        <x:v>Falcon</x:v>
       </x:c>
       <x:c r="AF147" t="str">
-        <x:v>Associação Atlética Guarany</x:v>
+        <x:v>Falcon Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="148">
       <x:c r="A148" t="str">
-        <x:v>SP</x:v>
+        <x:v>SE</x:v>
       </x:c>
       <x:c r="B148" t="str">
-        <x:v>Capivari</x:v>
+        <x:v>Porto da Folha</x:v>
       </x:c>
       <x:c r="C148"/>
       <x:c r="D148" t="str">
@@ -12875,10 +12873,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G148" t="str">
-        <x:v>Capivariano</x:v>
+        <x:v>Guarany de Porto da Folha</x:v>
       </x:c>
       <x:c r="H148" t="str">
-        <x:v>capivariano.png</x:v>
+        <x:v>guarany_de_porto_da_folha.png</x:v>
       </x:c>
       <x:c r="I148" t="str">
         <x:v>PNG</x:v>
@@ -12894,12 +12892,14 @@
       <x:c r="N148" t="str">
         <x:v>Football Kit Archive</x:v>
       </x:c>
-      <x:c r="O148"/>
+      <x:c r="O148" t="str">
+        <x:v>https://www.footballkitarchive.com/pt/campeonato-sergipano-kits/</x:v>
+      </x:c>
       <x:c r="P148" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Capivariano%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Guarany+de+Porto+da+Folha%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q148" t="str">
-        <x:v>PENDENTE DE FOTO DIRETA</x:v>
+        <x:v>REFERÊNCIA 2026 - COMPETIÇÃO</x:v>
       </x:c>
       <x:c r="R148" t="str">
         <x:v>Vermelho / Branco</x:v>
@@ -12935,10 +12935,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE148" t="str">
-        <x:v>Capivariano</x:v>
+        <x:v>Guarany de Porto da Folha</x:v>
       </x:c>
       <x:c r="AF148" t="str">
-        <x:v>Capivariano Futebol Clube</x:v>
+        <x:v>Associação Atlética Guarany</x:v>
       </x:c>
     </x:row>
     <x:row r="149">
@@ -12946,25 +12946,21 @@
         <x:v>SP</x:v>
       </x:c>
       <x:c r="B149" t="str">
-        <x:v>Bauru</x:v>
-      </x:c>
-      <x:c r="C149" t="str">
-        <x:v>D</x:v>
-      </x:c>
+        <x:v>Capivari</x:v>
+      </x:c>
+      <x:c r="C149"/>
       <x:c r="D149" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E149" t="str">
-        <x:v>Uniforme 2026 confirmado: Physicus; modelo lisa.</x:v>
-      </x:c>
+      <x:c r="E149"/>
       <x:c r="F149" t="str">
-        <x:v>D</x:v>
+        <x:v>estadual</x:v>
       </x:c>
       <x:c r="G149" t="str">
-        <x:v>Noroeste</x:v>
+        <x:v>Capivariano</x:v>
       </x:c>
       <x:c r="H149" t="str">
-        <x:v>noroeste.png</x:v>
+        <x:v>capivariano.png</x:v>
       </x:c>
       <x:c r="I149" t="str">
         <x:v>PNG</x:v>
@@ -12982,7 +12978,7 @@
       </x:c>
       <x:c r="O149"/>
       <x:c r="P149" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Noroeste%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Capivariano%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q149" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
@@ -13018,13 +13014,13 @@
       <x:c r="AB149"/>
       <x:c r="AC149"/>
       <x:c r="AD149" t="str">
-        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
+        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE149" t="str">
-        <x:v>Noroeste</x:v>
+        <x:v>Capivariano</x:v>
       </x:c>
       <x:c r="AF149" t="str">
-        <x:v>Esporte Clube Noroeste SAF</x:v>
+        <x:v>Capivariano Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="150">
@@ -13032,21 +13028,25 @@
         <x:v>SP</x:v>
       </x:c>
       <x:c r="B150" t="str">
-        <x:v>Indaiatuba</x:v>
-      </x:c>
-      <x:c r="C150"/>
+        <x:v>Bauru</x:v>
+      </x:c>
+      <x:c r="C150" t="str">
+        <x:v>D</x:v>
+      </x:c>
       <x:c r="D150" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E150"/>
+      <x:c r="E150" t="str">
+        <x:v>Uniforme 2026 confirmado: Physicus; modelo lisa.</x:v>
+      </x:c>
       <x:c r="F150" t="str">
-        <x:v>estadual</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="G150" t="str">
-        <x:v>Primavera-SP</x:v>
+        <x:v>Noroeste</x:v>
       </x:c>
       <x:c r="H150" t="str">
-        <x:v>primavera_sp.png</x:v>
+        <x:v>noroeste.png</x:v>
       </x:c>
       <x:c r="I150" t="str">
         <x:v>PNG</x:v>
@@ -13064,7 +13064,7 @@
       </x:c>
       <x:c r="O150"/>
       <x:c r="P150" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Primavera-SP%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Noroeste%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q150" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
@@ -13100,13 +13100,13 @@
       <x:c r="AB150"/>
       <x:c r="AC150"/>
       <x:c r="AD150" t="str">
-        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE150" t="str">
-        <x:v>Primavera-SP</x:v>
+        <x:v>Noroeste</x:v>
       </x:c>
       <x:c r="AF150" t="str">
-        <x:v>Esporte Clube Primavera</x:v>
+        <x:v>Esporte Clube Noroeste SAF</x:v>
       </x:c>
     </x:row>
     <x:row r="151">
@@ -13114,25 +13114,21 @@
         <x:v>SP</x:v>
       </x:c>
       <x:c r="B151" t="str">
-        <x:v>Rio Claro</x:v>
-      </x:c>
-      <x:c r="C151" t="str">
-        <x:v>D</x:v>
-      </x:c>
+        <x:v>Indaiatuba</x:v>
+      </x:c>
+      <x:c r="C151"/>
       <x:c r="D151" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E151" t="str">
-        <x:v>Uniforme 2026 confirmado: Junpe; modelo lisa.</x:v>
-      </x:c>
+      <x:c r="E151"/>
       <x:c r="F151" t="str">
-        <x:v>D</x:v>
+        <x:v>estadual</x:v>
       </x:c>
       <x:c r="G151" t="str">
-        <x:v>Velo Clube</x:v>
+        <x:v>Primavera-SP</x:v>
       </x:c>
       <x:c r="H151" t="str">
-        <x:v>velo_clube.png</x:v>
+        <x:v>primavera_sp.png</x:v>
       </x:c>
       <x:c r="I151" t="str">
         <x:v>PNG</x:v>
@@ -13150,19 +13146,19 @@
       </x:c>
       <x:c r="O151"/>
       <x:c r="P151" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Velo+Clube%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Primavera-SP%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q151" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R151" t="str">
-        <x:v>Vermelho / Verde</x:v>
+        <x:v>Vermelho / Branco</x:v>
       </x:c>
       <x:c r="S151" t="str">
-        <x:v>#D2232A / #00843D</x:v>
+        <x:v>#D2232A / #FFFFFF</x:v>
       </x:c>
       <x:c r="T151" t="str">
-        <x:v>210,35,42 / 0,132,61</x:v>
+        <x:v>210,35,42 / 255,255,255</x:v>
       </x:c>
       <x:c r="U151" t="str">
         <x:v>Vermelho</x:v>
@@ -13174,25 +13170,25 @@
         <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="X151" t="str">
-        <x:v>Verde</x:v>
+        <x:v>Branco</x:v>
       </x:c>
       <x:c r="Y151" t="str">
-        <x:v>#00843D</x:v>
+        <x:v>#FFFFFF</x:v>
       </x:c>
       <x:c r="Z151" t="str">
-        <x:v>0,132,61</x:v>
+        <x:v>255,255,255</x:v>
       </x:c>
       <x:c r="AA151"/>
       <x:c r="AB151"/>
       <x:c r="AC151"/>
       <x:c r="AD151" t="str">
-        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
+        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE151" t="str">
-        <x:v>Velo Clube</x:v>
+        <x:v>Primavera-SP</x:v>
       </x:c>
       <x:c r="AF151" t="str">
-        <x:v>Associação Esportiva Velo Clube Rioclarense</x:v>
+        <x:v>Esporte Clube Primavera</x:v>
       </x:c>
     </x:row>
     <x:row r="152">
@@ -13200,25 +13196,25 @@
         <x:v>SP</x:v>
       </x:c>
       <x:c r="B152" t="str">
-        <x:v>Piracicaba</x:v>
+        <x:v>Rio Claro</x:v>
       </x:c>
       <x:c r="C152" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="D152" t="str">
-        <x:v>não</x:v>
+        <x:v>sim</x:v>
       </x:c>
       <x:c r="E152" t="str">
-        <x:v>Uniforme 2026 confirmado: Kappa; modelo listras horizontais.</x:v>
+        <x:v>Uniforme 2026 confirmado: Junpe; modelo lisa.</x:v>
       </x:c>
       <x:c r="F152" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="G152" t="str">
-        <x:v>XV de Piracicaba</x:v>
+        <x:v>Velo Clube</x:v>
       </x:c>
       <x:c r="H152" t="str">
-        <x:v>xv_de_piracicaba.png</x:v>
+        <x:v>velo_clube.png</x:v>
       </x:c>
       <x:c r="I152" t="str">
         <x:v>PNG</x:v>
@@ -13236,37 +13232,37 @@
       </x:c>
       <x:c r="O152"/>
       <x:c r="P152" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22XV+de+Piracicaba%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Velo+Clube%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q152" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R152" t="str">
-        <x:v>Preto / Branco</x:v>
+        <x:v>Vermelho / Verde</x:v>
       </x:c>
       <x:c r="S152" t="str">
-        <x:v>#000000 / #FFFFFF</x:v>
+        <x:v>#D2232A / #00843D</x:v>
       </x:c>
       <x:c r="T152" t="str">
-        <x:v>0,0,0 / 255,255,255</x:v>
+        <x:v>210,35,42 / 0,132,61</x:v>
       </x:c>
       <x:c r="U152" t="str">
-        <x:v>Preto</x:v>
+        <x:v>Vermelho</x:v>
       </x:c>
       <x:c r="V152" t="str">
-        <x:v>#000000</x:v>
+        <x:v>#D2232A</x:v>
       </x:c>
       <x:c r="W152" t="str">
-        <x:v>0,0,0</x:v>
+        <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="X152" t="str">
-        <x:v>Branco</x:v>
+        <x:v>Verde</x:v>
       </x:c>
       <x:c r="Y152" t="str">
-        <x:v>#FFFFFF</x:v>
+        <x:v>#00843D</x:v>
       </x:c>
       <x:c r="Z152" t="str">
-        <x:v>255,255,255</x:v>
+        <x:v>0,132,61</x:v>
       </x:c>
       <x:c r="AA152"/>
       <x:c r="AB152"/>
@@ -13275,36 +13271,36 @@
         <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE152" t="str">
-        <x:v>XV de Piracicaba</x:v>
+        <x:v>Velo Clube</x:v>
       </x:c>
       <x:c r="AF152" t="str">
-        <x:v>Esporte Clube XV de Novembro</x:v>
+        <x:v>Associação Esportiva Velo Clube Rioclarense</x:v>
       </x:c>
     </x:row>
     <x:row r="153">
       <x:c r="A153" t="str">
-        <x:v>TO</x:v>
+        <x:v>SP</x:v>
       </x:c>
       <x:c r="B153" t="str">
-        <x:v>Araguaína</x:v>
+        <x:v>Piracicaba</x:v>
       </x:c>
       <x:c r="C153" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="D153" t="str">
-        <x:v>sim</x:v>
+        <x:v>não</x:v>
       </x:c>
       <x:c r="E153" t="str">
-        <x:v>Uniforme 2026 confirmado: Likos; modelo listras verticais.</x:v>
+        <x:v>Uniforme 2026 confirmado: Kappa; modelo listras horizontais.</x:v>
       </x:c>
       <x:c r="F153" t="str">
         <x:v>D</x:v>
       </x:c>
       <x:c r="G153" t="str">
-        <x:v>Araguaína</x:v>
+        <x:v>XV de Piracicaba</x:v>
       </x:c>
       <x:c r="H153" t="str">
-        <x:v>araguaina.png</x:v>
+        <x:v>xv_de_piracicaba.png</x:v>
       </x:c>
       <x:c r="I153" t="str">
         <x:v>PNG</x:v>
@@ -13322,28 +13318,28 @@
       </x:c>
       <x:c r="O153"/>
       <x:c r="P153" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Aragua%C3%ADna%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22XV+de+Piracicaba%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q153" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R153" t="str">
-        <x:v>Vermelho / Branco / Azul</x:v>
+        <x:v>Preto / Branco</x:v>
       </x:c>
       <x:c r="S153" t="str">
-        <x:v>#D2232A / #FFFFFF / #0057B8</x:v>
+        <x:v>#000000 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T153" t="str">
-        <x:v>210,35,42 / 255,255,255 / 0,87,184</x:v>
+        <x:v>0,0,0 / 255,255,255</x:v>
       </x:c>
       <x:c r="U153" t="str">
-        <x:v>Vermelho</x:v>
+        <x:v>Preto</x:v>
       </x:c>
       <x:c r="V153" t="str">
-        <x:v>#D2232A</x:v>
+        <x:v>#000000</x:v>
       </x:c>
       <x:c r="W153" t="str">
-        <x:v>210,35,42</x:v>
+        <x:v>0,0,0</x:v>
       </x:c>
       <x:c r="X153" t="str">
         <x:v>Branco</x:v>
@@ -13354,23 +13350,17 @@
       <x:c r="Z153" t="str">
         <x:v>255,255,255</x:v>
       </x:c>
-      <x:c r="AA153" t="str">
-        <x:v>Azul</x:v>
-      </x:c>
-      <x:c r="AB153" t="str">
-        <x:v>#0057B8</x:v>
-      </x:c>
-      <x:c r="AC153" t="str">
-        <x:v>0,87,184</x:v>
-      </x:c>
+      <x:c r="AA153"/>
+      <x:c r="AB153"/>
+      <x:c r="AC153"/>
       <x:c r="AD153" t="str">
         <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE153" t="str">
-        <x:v>Araguaína</x:v>
+        <x:v>XV de Piracicaba</x:v>
       </x:c>
       <x:c r="AF153" t="str">
-        <x:v>Araguaína Futebol e Regatas</x:v>
+        <x:v>Esporte Clube XV de Novembro</x:v>
       </x:c>
     </x:row>
     <x:row r="154">
@@ -13378,21 +13368,25 @@
         <x:v>TO</x:v>
       </x:c>
       <x:c r="B154" t="str">
-        <x:v>Cachoeirinha</x:v>
-      </x:c>
-      <x:c r="C154"/>
+        <x:v>Araguaína</x:v>
+      </x:c>
+      <x:c r="C154" t="str">
+        <x:v>D</x:v>
+      </x:c>
       <x:c r="D154" t="str">
         <x:v>sim</x:v>
       </x:c>
-      <x:c r="E154"/>
+      <x:c r="E154" t="str">
+        <x:v>Uniforme 2026 confirmado: Likos; modelo listras verticais.</x:v>
+      </x:c>
       <x:c r="F154" t="str">
-        <x:v>estadual</x:v>
+        <x:v>D</x:v>
       </x:c>
       <x:c r="G154" t="str">
-        <x:v>Bela Vista</x:v>
+        <x:v>Araguaína</x:v>
       </x:c>
       <x:c r="H154" t="str">
-        <x:v>bela_vista.png</x:v>
+        <x:v>araguaina.png</x:v>
       </x:c>
       <x:c r="I154" t="str">
         <x:v>PNG</x:v>
@@ -13410,28 +13404,28 @@
       </x:c>
       <x:c r="O154"/>
       <x:c r="P154" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Bela+Vista%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Aragua%C3%ADna%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q154" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R154" t="str">
-        <x:v>Azul / Branco</x:v>
+        <x:v>Vermelho / Branco / Azul</x:v>
       </x:c>
       <x:c r="S154" t="str">
-        <x:v>#0057B8 / #FFFFFF</x:v>
+        <x:v>#D2232A / #FFFFFF / #0057B8</x:v>
       </x:c>
       <x:c r="T154" t="str">
-        <x:v>0,87,184 / 255,255,255</x:v>
+        <x:v>210,35,42 / 255,255,255 / 0,87,184</x:v>
       </x:c>
       <x:c r="U154" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Vermelho</x:v>
       </x:c>
       <x:c r="V154" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#D2232A</x:v>
       </x:c>
       <x:c r="W154" t="str">
-        <x:v>0,87,184</x:v>
+        <x:v>210,35,42</x:v>
       </x:c>
       <x:c r="X154" t="str">
         <x:v>Branco</x:v>
@@ -13442,17 +13436,23 @@
       <x:c r="Z154" t="str">
         <x:v>255,255,255</x:v>
       </x:c>
-      <x:c r="AA154"/>
-      <x:c r="AB154"/>
-      <x:c r="AC154"/>
+      <x:c r="AA154" t="str">
+        <x:v>Azul</x:v>
+      </x:c>
+      <x:c r="AB154" t="str">
+        <x:v>#0057B8</x:v>
+      </x:c>
+      <x:c r="AC154" t="str">
+        <x:v>0,87,184</x:v>
+      </x:c>
       <x:c r="AD154" t="str">
-        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+        <x:v>Football Kit Archive 2026 (uniforme titular)</x:v>
       </x:c>
       <x:c r="AE154" t="str">
-        <x:v>Bela Vista</x:v>
+        <x:v>Araguaína</x:v>
       </x:c>
       <x:c r="AF154" t="str">
-        <x:v>Instituto Bela Vista Futebol Cachoeirense</x:v>
+        <x:v>Araguaína Futebol e Regatas</x:v>
       </x:c>
     </x:row>
     <x:row r="155">
@@ -13460,7 +13460,7 @@
         <x:v>TO</x:v>
       </x:c>
       <x:c r="B155" t="str">
-        <x:v>Palmas</x:v>
+        <x:v>Cachoeirinha</x:v>
       </x:c>
       <x:c r="C155"/>
       <x:c r="D155" t="str">
@@ -13471,10 +13471,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G155" t="str">
-        <x:v>Capital-TO</x:v>
+        <x:v>Bela Vista</x:v>
       </x:c>
       <x:c r="H155" t="str">
-        <x:v>capital_to.png</x:v>
+        <x:v>bela_vista.png</x:v>
       </x:c>
       <x:c r="I155" t="str">
         <x:v>PNG</x:v>
@@ -13492,7 +13492,7 @@
       </x:c>
       <x:c r="O155"/>
       <x:c r="P155" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Capital-TO%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Bela+Vista%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q155" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
@@ -13531,10 +13531,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE155" t="str">
-        <x:v>Capital-TO</x:v>
+        <x:v>Bela Vista</x:v>
       </x:c>
       <x:c r="AF155" t="str">
-        <x:v>Capital Futebol Clube</x:v>
+        <x:v>Instituto Bela Vista Futebol Cachoeirense</x:v>
       </x:c>
     </x:row>
     <x:row r="156">
@@ -13542,7 +13542,7 @@
         <x:v>TO</x:v>
       </x:c>
       <x:c r="B156" t="str">
-        <x:v>Guaraí</x:v>
+        <x:v>Palmas</x:v>
       </x:c>
       <x:c r="C156"/>
       <x:c r="D156" t="str">
@@ -13553,10 +13553,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G156" t="str">
-        <x:v>Guaraí</x:v>
+        <x:v>Capital-TO</x:v>
       </x:c>
       <x:c r="H156" t="str">
-        <x:v>guarai.png</x:v>
+        <x:v>capital_to.png</x:v>
       </x:c>
       <x:c r="I156" t="str">
         <x:v>PNG</x:v>
@@ -13574,7 +13574,7 @@
       </x:c>
       <x:c r="O156"/>
       <x:c r="P156" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Guara%C3%AD%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Capital-TO%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q156" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
@@ -13613,10 +13613,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE156" t="str">
-        <x:v>Guaraí</x:v>
+        <x:v>Capital-TO</x:v>
       </x:c>
       <x:c r="AF156" t="str">
-        <x:v>Sport Club Guaraí</x:v>
+        <x:v>Capital Futebol Clube</x:v>
       </x:c>
     </x:row>
     <x:row r="157">
@@ -13624,7 +13624,7 @@
         <x:v>TO</x:v>
       </x:c>
       <x:c r="B157" t="str">
-        <x:v>Gurupi</x:v>
+        <x:v>Guaraí</x:v>
       </x:c>
       <x:c r="C157"/>
       <x:c r="D157" t="str">
@@ -13635,10 +13635,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G157" t="str">
-        <x:v>Gurupi</x:v>
+        <x:v>Guaraí</x:v>
       </x:c>
       <x:c r="H157" t="str">
-        <x:v>gurupi.png</x:v>
+        <x:v>guarai.png</x:v>
       </x:c>
       <x:c r="I157" t="str">
         <x:v>PNG</x:v>
@@ -13656,28 +13656,28 @@
       </x:c>
       <x:c r="O157"/>
       <x:c r="P157" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Gurupi%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Guara%C3%AD%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q157" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R157" t="str">
-        <x:v>Verde / Branco</x:v>
+        <x:v>Azul / Branco</x:v>
       </x:c>
       <x:c r="S157" t="str">
-        <x:v>#00843D / #FFFFFF</x:v>
+        <x:v>#0057B8 / #FFFFFF</x:v>
       </x:c>
       <x:c r="T157" t="str">
-        <x:v>0,132,61 / 255,255,255</x:v>
+        <x:v>0,87,184 / 255,255,255</x:v>
       </x:c>
       <x:c r="U157" t="str">
-        <x:v>Verde</x:v>
+        <x:v>Azul</x:v>
       </x:c>
       <x:c r="V157" t="str">
-        <x:v>#00843D</x:v>
+        <x:v>#0057B8</x:v>
       </x:c>
       <x:c r="W157" t="str">
-        <x:v>0,132,61</x:v>
+        <x:v>0,87,184</x:v>
       </x:c>
       <x:c r="X157" t="str">
         <x:v>Branco</x:v>
@@ -13695,10 +13695,10 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE157" t="str">
-        <x:v>Gurupi</x:v>
+        <x:v>Guaraí</x:v>
       </x:c>
       <x:c r="AF157" t="str">
-        <x:v>Gurupi Esporte Clube</x:v>
+        <x:v>Sport Club Guaraí</x:v>
       </x:c>
     </x:row>
     <x:row r="158">
@@ -13706,7 +13706,7 @@
         <x:v>TO</x:v>
       </x:c>
       <x:c r="B158" t="str">
-        <x:v>Palmas</x:v>
+        <x:v>Gurupi</x:v>
       </x:c>
       <x:c r="C158"/>
       <x:c r="D158" t="str">
@@ -13717,10 +13717,10 @@
         <x:v>estadual</x:v>
       </x:c>
       <x:c r="G158" t="str">
-        <x:v>Palmas</x:v>
+        <x:v>Gurupi</x:v>
       </x:c>
       <x:c r="H158" t="str">
-        <x:v>palmas.png</x:v>
+        <x:v>gurupi.png</x:v>
       </x:c>
       <x:c r="I158" t="str">
         <x:v>PNG</x:v>
@@ -13738,28 +13738,28 @@
       </x:c>
       <x:c r="O158"/>
       <x:c r="P158" t="str">
-        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Palmas%22+%222026%22+kit</x:v>
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Gurupi%22+%222026%22+kit</x:v>
       </x:c>
       <x:c r="Q158" t="str">
         <x:v>PENDENTE DE FOTO DIRETA</x:v>
       </x:c>
       <x:c r="R158" t="str">
-        <x:v>Azul / Branco</x:v>
+        <x:v>Verde / Branco</x:v>
       </x:c>
       <x:c r="S158" t="str">
-        <x:v>#0057B8 / #FFFFFF</x:v>
+        <x:v>#00843D / #FFFFFF</x:v>
       </x:c>
       <x:c r="T158" t="str">
-        <x:v>0,87,184 / 255,255,255</x:v>
+        <x:v>0,132,61 / 255,255,255</x:v>
       </x:c>
       <x:c r="U158" t="str">
-        <x:v>Azul</x:v>
+        <x:v>Verde</x:v>
       </x:c>
       <x:c r="V158" t="str">
-        <x:v>#0057B8</x:v>
+        <x:v>#00843D</x:v>
       </x:c>
       <x:c r="W158" t="str">
-        <x:v>0,87,184</x:v>
+        <x:v>0,132,61</x:v>
       </x:c>
       <x:c r="X158" t="str">
         <x:v>Branco</x:v>
@@ -13777,45 +13777,93 @@
         <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
       </x:c>
       <x:c r="AE158" t="str">
+        <x:v>Gurupi</x:v>
+      </x:c>
+      <x:c r="AF158" t="str">
+        <x:v>Gurupi Esporte Clube</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="159">
+      <x:c r="A159" t="str">
+        <x:v>TO</x:v>
+      </x:c>
+      <x:c r="B159" t="str">
         <x:v>Palmas</x:v>
       </x:c>
-      <x:c r="AF158" t="str">
-        <x:v>Palmas Futebol e Regatas</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="159">
-      <x:c r="A159"/>
-      <x:c r="B159"/>
       <x:c r="C159"/>
-      <x:c r="D159"/>
+      <x:c r="D159" t="str">
+        <x:v>sim</x:v>
+      </x:c>
       <x:c r="E159"/>
-      <x:c r="F159"/>
-      <x:c r="G159"/>
-      <x:c r="H159"/>
-      <x:c r="I159"/>
+      <x:c r="F159" t="str">
+        <x:v>estadual</x:v>
+      </x:c>
+      <x:c r="G159" t="str">
+        <x:v>Palmas</x:v>
+      </x:c>
+      <x:c r="H159" t="str">
+        <x:v>palmas.png</x:v>
+      </x:c>
+      <x:c r="I159" t="str">
+        <x:v>PNG</x:v>
+      </x:c>
       <x:c r="J159"/>
       <x:c r="K159"/>
-      <x:c r="L159"/>
-      <x:c r="M159"/>
-      <x:c r="N159"/>
+      <x:c r="L159" t="str">
+        <x:v>PENDENTE DE DOWNLOAD</x:v>
+      </x:c>
+      <x:c r="M159" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="N159" t="str">
+        <x:v>Football Kit Archive</x:v>
+      </x:c>
       <x:c r="O159"/>
-      <x:c r="P159"/>
-      <x:c r="Q159"/>
-      <x:c r="R159"/>
-      <x:c r="S159"/>
-      <x:c r="T159"/>
-      <x:c r="U159"/>
-      <x:c r="V159"/>
-      <x:c r="W159"/>
-      <x:c r="X159"/>
-      <x:c r="Y159"/>
-      <x:c r="Z159"/>
+      <x:c r="P159" t="str">
+        <x:v>https://www.google.com/search?q=site%3Afootballkitarchive.com+%22Palmas%22+%222026%22+kit</x:v>
+      </x:c>
+      <x:c r="Q159" t="str">
+        <x:v>PENDENTE DE FOTO DIRETA</x:v>
+      </x:c>
+      <x:c r="R159" t="str">
+        <x:v>Azul / Branco</x:v>
+      </x:c>
+      <x:c r="S159" t="str">
+        <x:v>#0057B8 / #FFFFFF</x:v>
+      </x:c>
+      <x:c r="T159" t="str">
+        <x:v>0,87,184 / 255,255,255</x:v>
+      </x:c>
+      <x:c r="U159" t="str">
+        <x:v>Azul</x:v>
+      </x:c>
+      <x:c r="V159" t="str">
+        <x:v>#0057B8</x:v>
+      </x:c>
+      <x:c r="W159" t="str">
+        <x:v>0,87,184</x:v>
+      </x:c>
+      <x:c r="X159" t="str">
+        <x:v>Branco</x:v>
+      </x:c>
+      <x:c r="Y159" t="str">
+        <x:v>#FFFFFF</x:v>
+      </x:c>
+      <x:c r="Z159" t="str">
+        <x:v>255,255,255</x:v>
+      </x:c>
       <x:c r="AA159"/>
       <x:c r="AB159"/>
       <x:c r="AC159"/>
-      <x:c r="AD159"/>
-      <x:c r="AE159"/>
-      <x:c r="AF159"/>
+      <x:c r="AD159" t="str">
+        <x:v>cores do clube / referência visual 2026; validar tonalidade final</x:v>
+      </x:c>
+      <x:c r="AE159" t="str">
+        <x:v>Palmas</x:v>
+      </x:c>
+      <x:c r="AF159" t="str">
+        <x:v>Palmas Futebol e Regatas</x:v>
+      </x:c>
     </x:row>
     <x:row r="160">
       <x:c r="A160"/>
@@ -13964,22 +14012,22 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>Clubes de 2026 ausentes do master: 157 linhas únicas após correção de duplicidades e entradas combinadas.</x:v>
+        <x:v>Clubes de 2026 ausentes do master: 158 linhas únicas após correção de duplicidades e entradas combinadas.</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Removidos: Cascavel, Decisão, Pantanal, PSTC/São Joseense e Parnamirim/ABC-D pelos motivos documentados na planilha de uniformes.</x:v>
+        <x:v>Parnamirim foi recolocado: é o Parnamirim Sport Clube, distinto do ABC. Em 2026 confirmou participação na 2ª divisão estadual, mas desistiu antes do início.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>São Joseense foi mantido como Independente Futebol São Joseense, distinto do PSTC, e marcado como Série D + estadual em 2026.</x:v>
+        <x:v>Removidos apenas os duplicados/entradas combinadas: Cascavel, Decisão, Pantanal, PSTC/São Joseense e Parnamirim/ABC-D; o clube correto Parnamirim permanece em linha própria.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Cores e referências de kit foram atualizadas com Football Kit Archive 2026 quando havia página confiável; dados não confirmados continuam pendentes em vez de serem inventados.</x:v>
+        <x:v>São Joseense permanece como Independente Futebol São Joseense, distinto do PSTC, e marcado como Série D + estadual em 2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">

</xml_diff>